<commit_message>
Integra motor completo com validacao por leitura e inicializador local unico
</commit_message>
<xml_diff>
--- a/templates/planilha_modelo_euler.xlsx
+++ b/templates/planilha_modelo_euler.xlsx
@@ -1,18 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="LEIA-ME" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="diario" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="combustivel" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="amostras" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="eventos" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="instrumentos" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LEIA-ME" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="diario" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="combustivel" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="amostras" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="eventos" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="instrumentos" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -297,6 +297,97 @@
       <text>
         <t>De onde vem o dado. Dados reais de clientes nunca entram no repositório. Valores: `sintetico`, `publico`, `real`.
 Unidade: —
+Opcional</t>
+      </text>
+    </comment>
+    <comment ref="V1" authorId="0" shapeId="0">
+      <text>
+        <t>Estado termodinâmico do vapor na linha medida. Se vazio, a EULER mantém a hipótese conservadora atual de vapor saturado seco e marca essa hipótese como assumida. Valores: `saturado_seco`, `umido`, `superaquecido`.
+Unidade: —
+Opcional</t>
+      </text>
+    </comment>
+    <comment ref="W1" authorId="0" shapeId="0">
+      <text>
+        <t>Temperatura do vapor quando o estado registrado é superaquecido.
+Unidade: °C
+Opcional</t>
+      </text>
+    </comment>
+    <comment ref="X1" authorId="0" shapeId="0">
+      <text>
+        <t>Título x do vapor úmido (0 a 1). Só é usado quando o estado registrado é umido.
+Unidade: fração
+Opcional</t>
+      </text>
+    </comment>
+    <comment ref="Y1" authorId="0" shapeId="0">
+      <text>
+        <t>Massa total purgada desde a leitura anterior. Sem massa medida, a EULER não converte duração em perda energética.
+Unidade: kg desde a leitura anterior
+Opcional</t>
+      </text>
+    </comment>
+    <comment ref="Z1" authorId="0" shapeId="0">
+      <text>
+        <t>Pressão no ponto de origem da purga (tambor/linha associada), usada na entalpia da purga.
+Unidade: bar manométrico
+Opcional</t>
+      </text>
+    </comment>
+    <comment ref="AA1" authorId="0" shapeId="0">
+      <text>
+        <t>Vazão de água de alimentação no ponto usado para avaliar o economizador.
+Unidade: t/h
+Opcional</t>
+      </text>
+    </comment>
+    <comment ref="AB1" authorId="0" shapeId="0">
+      <text>
+        <t>Pressão da água no economizador, no mesmo trecho das temperaturas de água.
+Unidade: bar manométrico
+Opcional</t>
+      </text>
+    </comment>
+    <comment ref="AC1" authorId="0" shapeId="0">
+      <text>
+        <t>Temperatura da água na entrada do economizador.
+Unidade: °C
+Opcional</t>
+      </text>
+    </comment>
+    <comment ref="AD1" authorId="0" shapeId="0">
+      <text>
+        <t>Temperatura da água na saída do economizador.
+Unidade: °C
+Opcional</t>
+      </text>
+    </comment>
+    <comment ref="AE1" authorId="0" shapeId="0">
+      <text>
+        <t>Temperatura dos gases na entrada do economizador.
+Unidade: °C
+Opcional</t>
+      </text>
+    </comment>
+    <comment ref="AF1" authorId="0" shapeId="0">
+      <text>
+        <t>Temperatura dos gases na saída do economizador.
+Unidade: °C
+Opcional</t>
+      </text>
+    </comment>
+    <comment ref="AG1" authorId="0" shapeId="0">
+      <text>
+        <t>Diferença de pressão no trecho de gases associado à análise de transferência.
+Unidade: mbar
+Opcional</t>
+      </text>
+    </comment>
+    <comment ref="AH1" authorId="0" shapeId="0">
+      <text>
+        <t>Alias de titulo_vapor_frac; normalizado com aviso. Se ambos forem informados, precisam coincidir.
+Unidade: fração
 Opcional</t>
       </text>
     </comment>
@@ -1023,7 +1114,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U500"/>
+  <dimension ref="A1:AH500"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -1047,6 +1138,19 @@
     <col width="14" customWidth="1" min="19" max="19"/>
     <col width="33" customWidth="1" min="20" max="20"/>
     <col width="15" customWidth="1" min="21" max="21"/>
+    <col width="16" customWidth="1" min="22" max="22"/>
+    <col width="14" customWidth="1" min="23" max="23"/>
+    <col width="21" customWidth="1" min="24" max="24"/>
+    <col width="18" customWidth="1" min="25" max="25"/>
+    <col width="19" customWidth="1" min="26" max="26"/>
+    <col width="23" customWidth="1" min="27" max="27"/>
+    <col width="22" customWidth="1" min="28" max="28"/>
+    <col width="24" customWidth="1" min="29" max="29"/>
+    <col width="22" customWidth="1" min="30" max="30"/>
+    <col width="25" customWidth="1" min="31" max="31"/>
+    <col width="23" customWidth="1" min="32" max="32"/>
+    <col width="17" customWidth="1" min="33" max="33"/>
+    <col width="16" customWidth="1" min="34" max="34"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1155,6 +1259,71 @@
           <t>origem_dado</t>
         </is>
       </c>
+      <c r="V1" s="3" t="inlineStr">
+        <is>
+          <t>estado_vapor</t>
+        </is>
+      </c>
+      <c r="W1" s="3" t="inlineStr">
+        <is>
+          <t>t_vapor_c</t>
+        </is>
+      </c>
+      <c r="X1" s="3" t="inlineStr">
+        <is>
+          <t>titulo_vapor_frac</t>
+        </is>
+      </c>
+      <c r="Y1" s="3" t="inlineStr">
+        <is>
+          <t>massa_purga_kg</t>
+        </is>
+      </c>
+      <c r="Z1" s="3" t="inlineStr">
+        <is>
+          <t>p_purga_bar_man</t>
+        </is>
+      </c>
+      <c r="AA1" s="3" t="inlineStr">
+        <is>
+          <t>vazao_agua_alim_t_h</t>
+        </is>
+      </c>
+      <c r="AB1" s="3" t="inlineStr">
+        <is>
+          <t>p_agua_eco_bar_man</t>
+        </is>
+      </c>
+      <c r="AC1" s="3" t="inlineStr">
+        <is>
+          <t>t_agua_eco_entrada_c</t>
+        </is>
+      </c>
+      <c r="AD1" s="3" t="inlineStr">
+        <is>
+          <t>t_agua_eco_saida_c</t>
+        </is>
+      </c>
+      <c r="AE1" s="3" t="inlineStr">
+        <is>
+          <t>t_gases_eco_entrada_c</t>
+        </is>
+      </c>
+      <c r="AF1" s="3" t="inlineStr">
+        <is>
+          <t>t_gases_eco_saida_c</t>
+        </is>
+      </c>
+      <c r="AG1" s="3" t="inlineStr">
+        <is>
+          <t>dp_gases_mbar</t>
+        </is>
+      </c>
+      <c r="AH1" s="3" t="inlineStr">
+        <is>
+          <t>titulo_vapor</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
@@ -1233,6 +1402,7 @@
           <t>sintetico</t>
         </is>
       </c>
+      <c r="V2" s="4" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="4" t="n"/>
@@ -1247,6 +1417,7 @@
       <c r="S3" s="4" t="n"/>
       <c r="T3" s="4" t="n"/>
       <c r="U3" s="4" t="n"/>
+      <c r="V3" s="4" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="4" t="n"/>
@@ -1261,6 +1432,7 @@
       <c r="S4" s="4" t="n"/>
       <c r="T4" s="4" t="n"/>
       <c r="U4" s="4" t="n"/>
+      <c r="V4" s="4" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="4" t="n"/>
@@ -1275,6 +1447,7 @@
       <c r="S5" s="4" t="n"/>
       <c r="T5" s="4" t="n"/>
       <c r="U5" s="4" t="n"/>
+      <c r="V5" s="4" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="4" t="n"/>
@@ -1289,6 +1462,7 @@
       <c r="S6" s="4" t="n"/>
       <c r="T6" s="4" t="n"/>
       <c r="U6" s="4" t="n"/>
+      <c r="V6" s="4" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="4" t="n"/>
@@ -1303,6 +1477,7 @@
       <c r="S7" s="4" t="n"/>
       <c r="T7" s="4" t="n"/>
       <c r="U7" s="4" t="n"/>
+      <c r="V7" s="4" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="4" t="n"/>
@@ -1317,6 +1492,7 @@
       <c r="S8" s="4" t="n"/>
       <c r="T8" s="4" t="n"/>
       <c r="U8" s="4" t="n"/>
+      <c r="V8" s="4" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="4" t="n"/>
@@ -1331,6 +1507,7 @@
       <c r="S9" s="4" t="n"/>
       <c r="T9" s="4" t="n"/>
       <c r="U9" s="4" t="n"/>
+      <c r="V9" s="4" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="4" t="n"/>
@@ -1345,6 +1522,7 @@
       <c r="S10" s="4" t="n"/>
       <c r="T10" s="4" t="n"/>
       <c r="U10" s="4" t="n"/>
+      <c r="V10" s="4" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="4" t="n"/>
@@ -1359,6 +1537,7 @@
       <c r="S11" s="4" t="n"/>
       <c r="T11" s="4" t="n"/>
       <c r="U11" s="4" t="n"/>
+      <c r="V11" s="4" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="4" t="n"/>
@@ -1373,6 +1552,7 @@
       <c r="S12" s="4" t="n"/>
       <c r="T12" s="4" t="n"/>
       <c r="U12" s="4" t="n"/>
+      <c r="V12" s="4" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="4" t="n"/>
@@ -1387,6 +1567,7 @@
       <c r="S13" s="4" t="n"/>
       <c r="T13" s="4" t="n"/>
       <c r="U13" s="4" t="n"/>
+      <c r="V13" s="4" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="4" t="n"/>
@@ -1401,6 +1582,7 @@
       <c r="S14" s="4" t="n"/>
       <c r="T14" s="4" t="n"/>
       <c r="U14" s="4" t="n"/>
+      <c r="V14" s="4" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="4" t="n"/>
@@ -1415,6 +1597,7 @@
       <c r="S15" s="4" t="n"/>
       <c r="T15" s="4" t="n"/>
       <c r="U15" s="4" t="n"/>
+      <c r="V15" s="4" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="4" t="n"/>
@@ -1429,6 +1612,7 @@
       <c r="S16" s="4" t="n"/>
       <c r="T16" s="4" t="n"/>
       <c r="U16" s="4" t="n"/>
+      <c r="V16" s="4" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="4" t="n"/>
@@ -1443,6 +1627,7 @@
       <c r="S17" s="4" t="n"/>
       <c r="T17" s="4" t="n"/>
       <c r="U17" s="4" t="n"/>
+      <c r="V17" s="4" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="4" t="n"/>
@@ -1457,6 +1642,7 @@
       <c r="S18" s="4" t="n"/>
       <c r="T18" s="4" t="n"/>
       <c r="U18" s="4" t="n"/>
+      <c r="V18" s="4" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="4" t="n"/>
@@ -1471,6 +1657,7 @@
       <c r="S19" s="4" t="n"/>
       <c r="T19" s="4" t="n"/>
       <c r="U19" s="4" t="n"/>
+      <c r="V19" s="4" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="4" t="n"/>
@@ -1485,6 +1672,7 @@
       <c r="S20" s="4" t="n"/>
       <c r="T20" s="4" t="n"/>
       <c r="U20" s="4" t="n"/>
+      <c r="V20" s="4" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="4" t="n"/>
@@ -1499,6 +1687,7 @@
       <c r="S21" s="4" t="n"/>
       <c r="T21" s="4" t="n"/>
       <c r="U21" s="4" t="n"/>
+      <c r="V21" s="4" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="4" t="n"/>
@@ -1513,6 +1702,7 @@
       <c r="S22" s="4" t="n"/>
       <c r="T22" s="4" t="n"/>
       <c r="U22" s="4" t="n"/>
+      <c r="V22" s="4" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="4" t="n"/>
@@ -1527,6 +1717,7 @@
       <c r="S23" s="4" t="n"/>
       <c r="T23" s="4" t="n"/>
       <c r="U23" s="4" t="n"/>
+      <c r="V23" s="4" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="4" t="n"/>
@@ -1541,6 +1732,7 @@
       <c r="S24" s="4" t="n"/>
       <c r="T24" s="4" t="n"/>
       <c r="U24" s="4" t="n"/>
+      <c r="V24" s="4" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="4" t="n"/>
@@ -1555,6 +1747,7 @@
       <c r="S25" s="4" t="n"/>
       <c r="T25" s="4" t="n"/>
       <c r="U25" s="4" t="n"/>
+      <c r="V25" s="4" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="4" t="n"/>
@@ -1569,6 +1762,7 @@
       <c r="S26" s="4" t="n"/>
       <c r="T26" s="4" t="n"/>
       <c r="U26" s="4" t="n"/>
+      <c r="V26" s="4" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="4" t="n"/>
@@ -1583,6 +1777,7 @@
       <c r="S27" s="4" t="n"/>
       <c r="T27" s="4" t="n"/>
       <c r="U27" s="4" t="n"/>
+      <c r="V27" s="4" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="4" t="n"/>
@@ -1597,6 +1792,7 @@
       <c r="S28" s="4" t="n"/>
       <c r="T28" s="4" t="n"/>
       <c r="U28" s="4" t="n"/>
+      <c r="V28" s="4" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="4" t="n"/>
@@ -1611,6 +1807,7 @@
       <c r="S29" s="4" t="n"/>
       <c r="T29" s="4" t="n"/>
       <c r="U29" s="4" t="n"/>
+      <c r="V29" s="4" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="4" t="n"/>
@@ -1625,6 +1822,7 @@
       <c r="S30" s="4" t="n"/>
       <c r="T30" s="4" t="n"/>
       <c r="U30" s="4" t="n"/>
+      <c r="V30" s="4" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="4" t="n"/>
@@ -1639,6 +1837,7 @@
       <c r="S31" s="4" t="n"/>
       <c r="T31" s="4" t="n"/>
       <c r="U31" s="4" t="n"/>
+      <c r="V31" s="4" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="4" t="n"/>
@@ -1653,6 +1852,7 @@
       <c r="S32" s="4" t="n"/>
       <c r="T32" s="4" t="n"/>
       <c r="U32" s="4" t="n"/>
+      <c r="V32" s="4" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="4" t="n"/>
@@ -1667,6 +1867,7 @@
       <c r="S33" s="4" t="n"/>
       <c r="T33" s="4" t="n"/>
       <c r="U33" s="4" t="n"/>
+      <c r="V33" s="4" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="4" t="n"/>
@@ -1681,6 +1882,7 @@
       <c r="S34" s="4" t="n"/>
       <c r="T34" s="4" t="n"/>
       <c r="U34" s="4" t="n"/>
+      <c r="V34" s="4" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="4" t="n"/>
@@ -1695,6 +1897,7 @@
       <c r="S35" s="4" t="n"/>
       <c r="T35" s="4" t="n"/>
       <c r="U35" s="4" t="n"/>
+      <c r="V35" s="4" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="4" t="n"/>
@@ -1709,6 +1912,7 @@
       <c r="S36" s="4" t="n"/>
       <c r="T36" s="4" t="n"/>
       <c r="U36" s="4" t="n"/>
+      <c r="V36" s="4" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="4" t="n"/>
@@ -1723,6 +1927,7 @@
       <c r="S37" s="4" t="n"/>
       <c r="T37" s="4" t="n"/>
       <c r="U37" s="4" t="n"/>
+      <c r="V37" s="4" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="4" t="n"/>
@@ -1737,6 +1942,7 @@
       <c r="S38" s="4" t="n"/>
       <c r="T38" s="4" t="n"/>
       <c r="U38" s="4" t="n"/>
+      <c r="V38" s="4" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="4" t="n"/>
@@ -1751,6 +1957,7 @@
       <c r="S39" s="4" t="n"/>
       <c r="T39" s="4" t="n"/>
       <c r="U39" s="4" t="n"/>
+      <c r="V39" s="4" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="4" t="n"/>
@@ -1765,6 +1972,7 @@
       <c r="S40" s="4" t="n"/>
       <c r="T40" s="4" t="n"/>
       <c r="U40" s="4" t="n"/>
+      <c r="V40" s="4" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="4" t="n"/>
@@ -1779,6 +1987,7 @@
       <c r="S41" s="4" t="n"/>
       <c r="T41" s="4" t="n"/>
       <c r="U41" s="4" t="n"/>
+      <c r="V41" s="4" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="4" t="n"/>
@@ -1793,6 +2002,7 @@
       <c r="S42" s="4" t="n"/>
       <c r="T42" s="4" t="n"/>
       <c r="U42" s="4" t="n"/>
+      <c r="V42" s="4" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="4" t="n"/>
@@ -1807,6 +2017,7 @@
       <c r="S43" s="4" t="n"/>
       <c r="T43" s="4" t="n"/>
       <c r="U43" s="4" t="n"/>
+      <c r="V43" s="4" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="4" t="n"/>
@@ -1821,6 +2032,7 @@
       <c r="S44" s="4" t="n"/>
       <c r="T44" s="4" t="n"/>
       <c r="U44" s="4" t="n"/>
+      <c r="V44" s="4" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="4" t="n"/>
@@ -1835,6 +2047,7 @@
       <c r="S45" s="4" t="n"/>
       <c r="T45" s="4" t="n"/>
       <c r="U45" s="4" t="n"/>
+      <c r="V45" s="4" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="4" t="n"/>
@@ -1849,6 +2062,7 @@
       <c r="S46" s="4" t="n"/>
       <c r="T46" s="4" t="n"/>
       <c r="U46" s="4" t="n"/>
+      <c r="V46" s="4" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="4" t="n"/>
@@ -1863,6 +2077,7 @@
       <c r="S47" s="4" t="n"/>
       <c r="T47" s="4" t="n"/>
       <c r="U47" s="4" t="n"/>
+      <c r="V47" s="4" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="4" t="n"/>
@@ -1877,6 +2092,7 @@
       <c r="S48" s="4" t="n"/>
       <c r="T48" s="4" t="n"/>
       <c r="U48" s="4" t="n"/>
+      <c r="V48" s="4" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="4" t="n"/>
@@ -1891,6 +2107,7 @@
       <c r="S49" s="4" t="n"/>
       <c r="T49" s="4" t="n"/>
       <c r="U49" s="4" t="n"/>
+      <c r="V49" s="4" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="4" t="n"/>
@@ -1905,6 +2122,7 @@
       <c r="S50" s="4" t="n"/>
       <c r="T50" s="4" t="n"/>
       <c r="U50" s="4" t="n"/>
+      <c r="V50" s="4" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="4" t="n"/>
@@ -1919,6 +2137,7 @@
       <c r="S51" s="4" t="n"/>
       <c r="T51" s="4" t="n"/>
       <c r="U51" s="4" t="n"/>
+      <c r="V51" s="4" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="4" t="n"/>
@@ -1933,6 +2152,7 @@
       <c r="S52" s="4" t="n"/>
       <c r="T52" s="4" t="n"/>
       <c r="U52" s="4" t="n"/>
+      <c r="V52" s="4" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="4" t="n"/>
@@ -1947,6 +2167,7 @@
       <c r="S53" s="4" t="n"/>
       <c r="T53" s="4" t="n"/>
       <c r="U53" s="4" t="n"/>
+      <c r="V53" s="4" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="4" t="n"/>
@@ -1961,6 +2182,7 @@
       <c r="S54" s="4" t="n"/>
       <c r="T54" s="4" t="n"/>
       <c r="U54" s="4" t="n"/>
+      <c r="V54" s="4" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="4" t="n"/>
@@ -1975,6 +2197,7 @@
       <c r="S55" s="4" t="n"/>
       <c r="T55" s="4" t="n"/>
       <c r="U55" s="4" t="n"/>
+      <c r="V55" s="4" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="4" t="n"/>
@@ -1989,6 +2212,7 @@
       <c r="S56" s="4" t="n"/>
       <c r="T56" s="4" t="n"/>
       <c r="U56" s="4" t="n"/>
+      <c r="V56" s="4" t="n"/>
     </row>
     <row r="57">
       <c r="A57" s="4" t="n"/>
@@ -2003,6 +2227,7 @@
       <c r="S57" s="4" t="n"/>
       <c r="T57" s="4" t="n"/>
       <c r="U57" s="4" t="n"/>
+      <c r="V57" s="4" t="n"/>
     </row>
     <row r="58">
       <c r="A58" s="4" t="n"/>
@@ -2017,6 +2242,7 @@
       <c r="S58" s="4" t="n"/>
       <c r="T58" s="4" t="n"/>
       <c r="U58" s="4" t="n"/>
+      <c r="V58" s="4" t="n"/>
     </row>
     <row r="59">
       <c r="A59" s="4" t="n"/>
@@ -2031,6 +2257,7 @@
       <c r="S59" s="4" t="n"/>
       <c r="T59" s="4" t="n"/>
       <c r="U59" s="4" t="n"/>
+      <c r="V59" s="4" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="4" t="n"/>
@@ -2045,6 +2272,7 @@
       <c r="S60" s="4" t="n"/>
       <c r="T60" s="4" t="n"/>
       <c r="U60" s="4" t="n"/>
+      <c r="V60" s="4" t="n"/>
     </row>
     <row r="61">
       <c r="A61" s="4" t="n"/>
@@ -2059,6 +2287,7 @@
       <c r="S61" s="4" t="n"/>
       <c r="T61" s="4" t="n"/>
       <c r="U61" s="4" t="n"/>
+      <c r="V61" s="4" t="n"/>
     </row>
     <row r="62">
       <c r="A62" s="4" t="n"/>
@@ -2073,6 +2302,7 @@
       <c r="S62" s="4" t="n"/>
       <c r="T62" s="4" t="n"/>
       <c r="U62" s="4" t="n"/>
+      <c r="V62" s="4" t="n"/>
     </row>
     <row r="63">
       <c r="A63" s="4" t="n"/>
@@ -2087,6 +2317,7 @@
       <c r="S63" s="4" t="n"/>
       <c r="T63" s="4" t="n"/>
       <c r="U63" s="4" t="n"/>
+      <c r="V63" s="4" t="n"/>
     </row>
     <row r="64">
       <c r="A64" s="4" t="n"/>
@@ -2101,6 +2332,7 @@
       <c r="S64" s="4" t="n"/>
       <c r="T64" s="4" t="n"/>
       <c r="U64" s="4" t="n"/>
+      <c r="V64" s="4" t="n"/>
     </row>
     <row r="65">
       <c r="A65" s="4" t="n"/>
@@ -2115,6 +2347,7 @@
       <c r="S65" s="4" t="n"/>
       <c r="T65" s="4" t="n"/>
       <c r="U65" s="4" t="n"/>
+      <c r="V65" s="4" t="n"/>
     </row>
     <row r="66">
       <c r="A66" s="4" t="n"/>
@@ -2129,6 +2362,7 @@
       <c r="S66" s="4" t="n"/>
       <c r="T66" s="4" t="n"/>
       <c r="U66" s="4" t="n"/>
+      <c r="V66" s="4" t="n"/>
     </row>
     <row r="67">
       <c r="A67" s="4" t="n"/>
@@ -2143,6 +2377,7 @@
       <c r="S67" s="4" t="n"/>
       <c r="T67" s="4" t="n"/>
       <c r="U67" s="4" t="n"/>
+      <c r="V67" s="4" t="n"/>
     </row>
     <row r="68">
       <c r="A68" s="4" t="n"/>
@@ -2157,6 +2392,7 @@
       <c r="S68" s="4" t="n"/>
       <c r="T68" s="4" t="n"/>
       <c r="U68" s="4" t="n"/>
+      <c r="V68" s="4" t="n"/>
     </row>
     <row r="69">
       <c r="A69" s="4" t="n"/>
@@ -2171,6 +2407,7 @@
       <c r="S69" s="4" t="n"/>
       <c r="T69" s="4" t="n"/>
       <c r="U69" s="4" t="n"/>
+      <c r="V69" s="4" t="n"/>
     </row>
     <row r="70">
       <c r="A70" s="4" t="n"/>
@@ -2185,6 +2422,7 @@
       <c r="S70" s="4" t="n"/>
       <c r="T70" s="4" t="n"/>
       <c r="U70" s="4" t="n"/>
+      <c r="V70" s="4" t="n"/>
     </row>
     <row r="71">
       <c r="A71" s="4" t="n"/>
@@ -2199,6 +2437,7 @@
       <c r="S71" s="4" t="n"/>
       <c r="T71" s="4" t="n"/>
       <c r="U71" s="4" t="n"/>
+      <c r="V71" s="4" t="n"/>
     </row>
     <row r="72">
       <c r="A72" s="4" t="n"/>
@@ -2213,6 +2452,7 @@
       <c r="S72" s="4" t="n"/>
       <c r="T72" s="4" t="n"/>
       <c r="U72" s="4" t="n"/>
+      <c r="V72" s="4" t="n"/>
     </row>
     <row r="73">
       <c r="A73" s="4" t="n"/>
@@ -2227,6 +2467,7 @@
       <c r="S73" s="4" t="n"/>
       <c r="T73" s="4" t="n"/>
       <c r="U73" s="4" t="n"/>
+      <c r="V73" s="4" t="n"/>
     </row>
     <row r="74">
       <c r="A74" s="4" t="n"/>
@@ -2241,6 +2482,7 @@
       <c r="S74" s="4" t="n"/>
       <c r="T74" s="4" t="n"/>
       <c r="U74" s="4" t="n"/>
+      <c r="V74" s="4" t="n"/>
     </row>
     <row r="75">
       <c r="A75" s="4" t="n"/>
@@ -2255,6 +2497,7 @@
       <c r="S75" s="4" t="n"/>
       <c r="T75" s="4" t="n"/>
       <c r="U75" s="4" t="n"/>
+      <c r="V75" s="4" t="n"/>
     </row>
     <row r="76">
       <c r="A76" s="4" t="n"/>
@@ -2269,6 +2512,7 @@
       <c r="S76" s="4" t="n"/>
       <c r="T76" s="4" t="n"/>
       <c r="U76" s="4" t="n"/>
+      <c r="V76" s="4" t="n"/>
     </row>
     <row r="77">
       <c r="A77" s="4" t="n"/>
@@ -2283,6 +2527,7 @@
       <c r="S77" s="4" t="n"/>
       <c r="T77" s="4" t="n"/>
       <c r="U77" s="4" t="n"/>
+      <c r="V77" s="4" t="n"/>
     </row>
     <row r="78">
       <c r="A78" s="4" t="n"/>
@@ -2297,6 +2542,7 @@
       <c r="S78" s="4" t="n"/>
       <c r="T78" s="4" t="n"/>
       <c r="U78" s="4" t="n"/>
+      <c r="V78" s="4" t="n"/>
     </row>
     <row r="79">
       <c r="A79" s="4" t="n"/>
@@ -2311,6 +2557,7 @@
       <c r="S79" s="4" t="n"/>
       <c r="T79" s="4" t="n"/>
       <c r="U79" s="4" t="n"/>
+      <c r="V79" s="4" t="n"/>
     </row>
     <row r="80">
       <c r="A80" s="4" t="n"/>
@@ -2325,6 +2572,7 @@
       <c r="S80" s="4" t="n"/>
       <c r="T80" s="4" t="n"/>
       <c r="U80" s="4" t="n"/>
+      <c r="V80" s="4" t="n"/>
     </row>
     <row r="81">
       <c r="A81" s="4" t="n"/>
@@ -2339,6 +2587,7 @@
       <c r="S81" s="4" t="n"/>
       <c r="T81" s="4" t="n"/>
       <c r="U81" s="4" t="n"/>
+      <c r="V81" s="4" t="n"/>
     </row>
     <row r="82">
       <c r="A82" s="4" t="n"/>
@@ -2353,6 +2602,7 @@
       <c r="S82" s="4" t="n"/>
       <c r="T82" s="4" t="n"/>
       <c r="U82" s="4" t="n"/>
+      <c r="V82" s="4" t="n"/>
     </row>
     <row r="83">
       <c r="A83" s="4" t="n"/>
@@ -2367,6 +2617,7 @@
       <c r="S83" s="4" t="n"/>
       <c r="T83" s="4" t="n"/>
       <c r="U83" s="4" t="n"/>
+      <c r="V83" s="4" t="n"/>
     </row>
     <row r="84">
       <c r="A84" s="4" t="n"/>
@@ -2381,6 +2632,7 @@
       <c r="S84" s="4" t="n"/>
       <c r="T84" s="4" t="n"/>
       <c r="U84" s="4" t="n"/>
+      <c r="V84" s="4" t="n"/>
     </row>
     <row r="85">
       <c r="A85" s="4" t="n"/>
@@ -2395,6 +2647,7 @@
       <c r="S85" s="4" t="n"/>
       <c r="T85" s="4" t="n"/>
       <c r="U85" s="4" t="n"/>
+      <c r="V85" s="4" t="n"/>
     </row>
     <row r="86">
       <c r="A86" s="4" t="n"/>
@@ -2409,6 +2662,7 @@
       <c r="S86" s="4" t="n"/>
       <c r="T86" s="4" t="n"/>
       <c r="U86" s="4" t="n"/>
+      <c r="V86" s="4" t="n"/>
     </row>
     <row r="87">
       <c r="A87" s="4" t="n"/>
@@ -2423,6 +2677,7 @@
       <c r="S87" s="4" t="n"/>
       <c r="T87" s="4" t="n"/>
       <c r="U87" s="4" t="n"/>
+      <c r="V87" s="4" t="n"/>
     </row>
     <row r="88">
       <c r="A88" s="4" t="n"/>
@@ -2437,6 +2692,7 @@
       <c r="S88" s="4" t="n"/>
       <c r="T88" s="4" t="n"/>
       <c r="U88" s="4" t="n"/>
+      <c r="V88" s="4" t="n"/>
     </row>
     <row r="89">
       <c r="A89" s="4" t="n"/>
@@ -2451,6 +2707,7 @@
       <c r="S89" s="4" t="n"/>
       <c r="T89" s="4" t="n"/>
       <c r="U89" s="4" t="n"/>
+      <c r="V89" s="4" t="n"/>
     </row>
     <row r="90">
       <c r="A90" s="4" t="n"/>
@@ -2465,6 +2722,7 @@
       <c r="S90" s="4" t="n"/>
       <c r="T90" s="4" t="n"/>
       <c r="U90" s="4" t="n"/>
+      <c r="V90" s="4" t="n"/>
     </row>
     <row r="91">
       <c r="A91" s="4" t="n"/>
@@ -2479,6 +2737,7 @@
       <c r="S91" s="4" t="n"/>
       <c r="T91" s="4" t="n"/>
       <c r="U91" s="4" t="n"/>
+      <c r="V91" s="4" t="n"/>
     </row>
     <row r="92">
       <c r="A92" s="4" t="n"/>
@@ -2493,6 +2752,7 @@
       <c r="S92" s="4" t="n"/>
       <c r="T92" s="4" t="n"/>
       <c r="U92" s="4" t="n"/>
+      <c r="V92" s="4" t="n"/>
     </row>
     <row r="93">
       <c r="A93" s="4" t="n"/>
@@ -2507,6 +2767,7 @@
       <c r="S93" s="4" t="n"/>
       <c r="T93" s="4" t="n"/>
       <c r="U93" s="4" t="n"/>
+      <c r="V93" s="4" t="n"/>
     </row>
     <row r="94">
       <c r="A94" s="4" t="n"/>
@@ -2521,6 +2782,7 @@
       <c r="S94" s="4" t="n"/>
       <c r="T94" s="4" t="n"/>
       <c r="U94" s="4" t="n"/>
+      <c r="V94" s="4" t="n"/>
     </row>
     <row r="95">
       <c r="A95" s="4" t="n"/>
@@ -2535,6 +2797,7 @@
       <c r="S95" s="4" t="n"/>
       <c r="T95" s="4" t="n"/>
       <c r="U95" s="4" t="n"/>
+      <c r="V95" s="4" t="n"/>
     </row>
     <row r="96">
       <c r="A96" s="4" t="n"/>
@@ -2549,6 +2812,7 @@
       <c r="S96" s="4" t="n"/>
       <c r="T96" s="4" t="n"/>
       <c r="U96" s="4" t="n"/>
+      <c r="V96" s="4" t="n"/>
     </row>
     <row r="97">
       <c r="A97" s="4" t="n"/>
@@ -2563,6 +2827,7 @@
       <c r="S97" s="4" t="n"/>
       <c r="T97" s="4" t="n"/>
       <c r="U97" s="4" t="n"/>
+      <c r="V97" s="4" t="n"/>
     </row>
     <row r="98">
       <c r="A98" s="4" t="n"/>
@@ -2577,6 +2842,7 @@
       <c r="S98" s="4" t="n"/>
       <c r="T98" s="4" t="n"/>
       <c r="U98" s="4" t="n"/>
+      <c r="V98" s="4" t="n"/>
     </row>
     <row r="99">
       <c r="A99" s="4" t="n"/>
@@ -2591,6 +2857,7 @@
       <c r="S99" s="4" t="n"/>
       <c r="T99" s="4" t="n"/>
       <c r="U99" s="4" t="n"/>
+      <c r="V99" s="4" t="n"/>
     </row>
     <row r="100">
       <c r="A100" s="4" t="n"/>
@@ -2605,6 +2872,7 @@
       <c r="S100" s="4" t="n"/>
       <c r="T100" s="4" t="n"/>
       <c r="U100" s="4" t="n"/>
+      <c r="V100" s="4" t="n"/>
     </row>
     <row r="101">
       <c r="A101" s="4" t="n"/>
@@ -2619,6 +2887,7 @@
       <c r="S101" s="4" t="n"/>
       <c r="T101" s="4" t="n"/>
       <c r="U101" s="4" t="n"/>
+      <c r="V101" s="4" t="n"/>
     </row>
     <row r="102">
       <c r="A102" s="4" t="n"/>
@@ -2633,6 +2902,7 @@
       <c r="S102" s="4" t="n"/>
       <c r="T102" s="4" t="n"/>
       <c r="U102" s="4" t="n"/>
+      <c r="V102" s="4" t="n"/>
     </row>
     <row r="103">
       <c r="A103" s="4" t="n"/>
@@ -2647,6 +2917,7 @@
       <c r="S103" s="4" t="n"/>
       <c r="T103" s="4" t="n"/>
       <c r="U103" s="4" t="n"/>
+      <c r="V103" s="4" t="n"/>
     </row>
     <row r="104">
       <c r="A104" s="4" t="n"/>
@@ -2661,6 +2932,7 @@
       <c r="S104" s="4" t="n"/>
       <c r="T104" s="4" t="n"/>
       <c r="U104" s="4" t="n"/>
+      <c r="V104" s="4" t="n"/>
     </row>
     <row r="105">
       <c r="A105" s="4" t="n"/>
@@ -2675,6 +2947,7 @@
       <c r="S105" s="4" t="n"/>
       <c r="T105" s="4" t="n"/>
       <c r="U105" s="4" t="n"/>
+      <c r="V105" s="4" t="n"/>
     </row>
     <row r="106">
       <c r="A106" s="4" t="n"/>
@@ -2689,6 +2962,7 @@
       <c r="S106" s="4" t="n"/>
       <c r="T106" s="4" t="n"/>
       <c r="U106" s="4" t="n"/>
+      <c r="V106" s="4" t="n"/>
     </row>
     <row r="107">
       <c r="A107" s="4" t="n"/>
@@ -2703,6 +2977,7 @@
       <c r="S107" s="4" t="n"/>
       <c r="T107" s="4" t="n"/>
       <c r="U107" s="4" t="n"/>
+      <c r="V107" s="4" t="n"/>
     </row>
     <row r="108">
       <c r="A108" s="4" t="n"/>
@@ -2717,6 +2992,7 @@
       <c r="S108" s="4" t="n"/>
       <c r="T108" s="4" t="n"/>
       <c r="U108" s="4" t="n"/>
+      <c r="V108" s="4" t="n"/>
     </row>
     <row r="109">
       <c r="A109" s="4" t="n"/>
@@ -2731,6 +3007,7 @@
       <c r="S109" s="4" t="n"/>
       <c r="T109" s="4" t="n"/>
       <c r="U109" s="4" t="n"/>
+      <c r="V109" s="4" t="n"/>
     </row>
     <row r="110">
       <c r="A110" s="4" t="n"/>
@@ -2745,6 +3022,7 @@
       <c r="S110" s="4" t="n"/>
       <c r="T110" s="4" t="n"/>
       <c r="U110" s="4" t="n"/>
+      <c r="V110" s="4" t="n"/>
     </row>
     <row r="111">
       <c r="A111" s="4" t="n"/>
@@ -2759,6 +3037,7 @@
       <c r="S111" s="4" t="n"/>
       <c r="T111" s="4" t="n"/>
       <c r="U111" s="4" t="n"/>
+      <c r="V111" s="4" t="n"/>
     </row>
     <row r="112">
       <c r="A112" s="4" t="n"/>
@@ -2773,6 +3052,7 @@
       <c r="S112" s="4" t="n"/>
       <c r="T112" s="4" t="n"/>
       <c r="U112" s="4" t="n"/>
+      <c r="V112" s="4" t="n"/>
     </row>
     <row r="113">
       <c r="A113" s="4" t="n"/>
@@ -2787,6 +3067,7 @@
       <c r="S113" s="4" t="n"/>
       <c r="T113" s="4" t="n"/>
       <c r="U113" s="4" t="n"/>
+      <c r="V113" s="4" t="n"/>
     </row>
     <row r="114">
       <c r="A114" s="4" t="n"/>
@@ -2801,6 +3082,7 @@
       <c r="S114" s="4" t="n"/>
       <c r="T114" s="4" t="n"/>
       <c r="U114" s="4" t="n"/>
+      <c r="V114" s="4" t="n"/>
     </row>
     <row r="115">
       <c r="A115" s="4" t="n"/>
@@ -2815,6 +3097,7 @@
       <c r="S115" s="4" t="n"/>
       <c r="T115" s="4" t="n"/>
       <c r="U115" s="4" t="n"/>
+      <c r="V115" s="4" t="n"/>
     </row>
     <row r="116">
       <c r="A116" s="4" t="n"/>
@@ -2829,6 +3112,7 @@
       <c r="S116" s="4" t="n"/>
       <c r="T116" s="4" t="n"/>
       <c r="U116" s="4" t="n"/>
+      <c r="V116" s="4" t="n"/>
     </row>
     <row r="117">
       <c r="A117" s="4" t="n"/>
@@ -2843,6 +3127,7 @@
       <c r="S117" s="4" t="n"/>
       <c r="T117" s="4" t="n"/>
       <c r="U117" s="4" t="n"/>
+      <c r="V117" s="4" t="n"/>
     </row>
     <row r="118">
       <c r="A118" s="4" t="n"/>
@@ -2857,6 +3142,7 @@
       <c r="S118" s="4" t="n"/>
       <c r="T118" s="4" t="n"/>
       <c r="U118" s="4" t="n"/>
+      <c r="V118" s="4" t="n"/>
     </row>
     <row r="119">
       <c r="A119" s="4" t="n"/>
@@ -2871,6 +3157,7 @@
       <c r="S119" s="4" t="n"/>
       <c r="T119" s="4" t="n"/>
       <c r="U119" s="4" t="n"/>
+      <c r="V119" s="4" t="n"/>
     </row>
     <row r="120">
       <c r="A120" s="4" t="n"/>
@@ -2885,6 +3172,7 @@
       <c r="S120" s="4" t="n"/>
       <c r="T120" s="4" t="n"/>
       <c r="U120" s="4" t="n"/>
+      <c r="V120" s="4" t="n"/>
     </row>
     <row r="121">
       <c r="A121" s="4" t="n"/>
@@ -2899,6 +3187,7 @@
       <c r="S121" s="4" t="n"/>
       <c r="T121" s="4" t="n"/>
       <c r="U121" s="4" t="n"/>
+      <c r="V121" s="4" t="n"/>
     </row>
     <row r="122">
       <c r="A122" s="4" t="n"/>
@@ -2913,6 +3202,7 @@
       <c r="S122" s="4" t="n"/>
       <c r="T122" s="4" t="n"/>
       <c r="U122" s="4" t="n"/>
+      <c r="V122" s="4" t="n"/>
     </row>
     <row r="123">
       <c r="A123" s="4" t="n"/>
@@ -2927,6 +3217,7 @@
       <c r="S123" s="4" t="n"/>
       <c r="T123" s="4" t="n"/>
       <c r="U123" s="4" t="n"/>
+      <c r="V123" s="4" t="n"/>
     </row>
     <row r="124">
       <c r="A124" s="4" t="n"/>
@@ -2941,6 +3232,7 @@
       <c r="S124" s="4" t="n"/>
       <c r="T124" s="4" t="n"/>
       <c r="U124" s="4" t="n"/>
+      <c r="V124" s="4" t="n"/>
     </row>
     <row r="125">
       <c r="A125" s="4" t="n"/>
@@ -2955,6 +3247,7 @@
       <c r="S125" s="4" t="n"/>
       <c r="T125" s="4" t="n"/>
       <c r="U125" s="4" t="n"/>
+      <c r="V125" s="4" t="n"/>
     </row>
     <row r="126">
       <c r="A126" s="4" t="n"/>
@@ -2969,6 +3262,7 @@
       <c r="S126" s="4" t="n"/>
       <c r="T126" s="4" t="n"/>
       <c r="U126" s="4" t="n"/>
+      <c r="V126" s="4" t="n"/>
     </row>
     <row r="127">
       <c r="A127" s="4" t="n"/>
@@ -2983,6 +3277,7 @@
       <c r="S127" s="4" t="n"/>
       <c r="T127" s="4" t="n"/>
       <c r="U127" s="4" t="n"/>
+      <c r="V127" s="4" t="n"/>
     </row>
     <row r="128">
       <c r="A128" s="4" t="n"/>
@@ -2997,6 +3292,7 @@
       <c r="S128" s="4" t="n"/>
       <c r="T128" s="4" t="n"/>
       <c r="U128" s="4" t="n"/>
+      <c r="V128" s="4" t="n"/>
     </row>
     <row r="129">
       <c r="A129" s="4" t="n"/>
@@ -3011,6 +3307,7 @@
       <c r="S129" s="4" t="n"/>
       <c r="T129" s="4" t="n"/>
       <c r="U129" s="4" t="n"/>
+      <c r="V129" s="4" t="n"/>
     </row>
     <row r="130">
       <c r="A130" s="4" t="n"/>
@@ -3025,6 +3322,7 @@
       <c r="S130" s="4" t="n"/>
       <c r="T130" s="4" t="n"/>
       <c r="U130" s="4" t="n"/>
+      <c r="V130" s="4" t="n"/>
     </row>
     <row r="131">
       <c r="A131" s="4" t="n"/>
@@ -3039,6 +3337,7 @@
       <c r="S131" s="4" t="n"/>
       <c r="T131" s="4" t="n"/>
       <c r="U131" s="4" t="n"/>
+      <c r="V131" s="4" t="n"/>
     </row>
     <row r="132">
       <c r="A132" s="4" t="n"/>
@@ -3053,6 +3352,7 @@
       <c r="S132" s="4" t="n"/>
       <c r="T132" s="4" t="n"/>
       <c r="U132" s="4" t="n"/>
+      <c r="V132" s="4" t="n"/>
     </row>
     <row r="133">
       <c r="A133" s="4" t="n"/>
@@ -3067,6 +3367,7 @@
       <c r="S133" s="4" t="n"/>
       <c r="T133" s="4" t="n"/>
       <c r="U133" s="4" t="n"/>
+      <c r="V133" s="4" t="n"/>
     </row>
     <row r="134">
       <c r="A134" s="4" t="n"/>
@@ -3081,6 +3382,7 @@
       <c r="S134" s="4" t="n"/>
       <c r="T134" s="4" t="n"/>
       <c r="U134" s="4" t="n"/>
+      <c r="V134" s="4" t="n"/>
     </row>
     <row r="135">
       <c r="A135" s="4" t="n"/>
@@ -3095,6 +3397,7 @@
       <c r="S135" s="4" t="n"/>
       <c r="T135" s="4" t="n"/>
       <c r="U135" s="4" t="n"/>
+      <c r="V135" s="4" t="n"/>
     </row>
     <row r="136">
       <c r="A136" s="4" t="n"/>
@@ -3109,6 +3412,7 @@
       <c r="S136" s="4" t="n"/>
       <c r="T136" s="4" t="n"/>
       <c r="U136" s="4" t="n"/>
+      <c r="V136" s="4" t="n"/>
     </row>
     <row r="137">
       <c r="A137" s="4" t="n"/>
@@ -3123,6 +3427,7 @@
       <c r="S137" s="4" t="n"/>
       <c r="T137" s="4" t="n"/>
       <c r="U137" s="4" t="n"/>
+      <c r="V137" s="4" t="n"/>
     </row>
     <row r="138">
       <c r="A138" s="4" t="n"/>
@@ -3137,6 +3442,7 @@
       <c r="S138" s="4" t="n"/>
       <c r="T138" s="4" t="n"/>
       <c r="U138" s="4" t="n"/>
+      <c r="V138" s="4" t="n"/>
     </row>
     <row r="139">
       <c r="A139" s="4" t="n"/>
@@ -3151,6 +3457,7 @@
       <c r="S139" s="4" t="n"/>
       <c r="T139" s="4" t="n"/>
       <c r="U139" s="4" t="n"/>
+      <c r="V139" s="4" t="n"/>
     </row>
     <row r="140">
       <c r="A140" s="4" t="n"/>
@@ -3165,6 +3472,7 @@
       <c r="S140" s="4" t="n"/>
       <c r="T140" s="4" t="n"/>
       <c r="U140" s="4" t="n"/>
+      <c r="V140" s="4" t="n"/>
     </row>
     <row r="141">
       <c r="A141" s="4" t="n"/>
@@ -3179,6 +3487,7 @@
       <c r="S141" s="4" t="n"/>
       <c r="T141" s="4" t="n"/>
       <c r="U141" s="4" t="n"/>
+      <c r="V141" s="4" t="n"/>
     </row>
     <row r="142">
       <c r="A142" s="4" t="n"/>
@@ -3193,6 +3502,7 @@
       <c r="S142" s="4" t="n"/>
       <c r="T142" s="4" t="n"/>
       <c r="U142" s="4" t="n"/>
+      <c r="V142" s="4" t="n"/>
     </row>
     <row r="143">
       <c r="A143" s="4" t="n"/>
@@ -3207,6 +3517,7 @@
       <c r="S143" s="4" t="n"/>
       <c r="T143" s="4" t="n"/>
       <c r="U143" s="4" t="n"/>
+      <c r="V143" s="4" t="n"/>
     </row>
     <row r="144">
       <c r="A144" s="4" t="n"/>
@@ -3221,6 +3532,7 @@
       <c r="S144" s="4" t="n"/>
       <c r="T144" s="4" t="n"/>
       <c r="U144" s="4" t="n"/>
+      <c r="V144" s="4" t="n"/>
     </row>
     <row r="145">
       <c r="A145" s="4" t="n"/>
@@ -3235,6 +3547,7 @@
       <c r="S145" s="4" t="n"/>
       <c r="T145" s="4" t="n"/>
       <c r="U145" s="4" t="n"/>
+      <c r="V145" s="4" t="n"/>
     </row>
     <row r="146">
       <c r="A146" s="4" t="n"/>
@@ -3249,6 +3562,7 @@
       <c r="S146" s="4" t="n"/>
       <c r="T146" s="4" t="n"/>
       <c r="U146" s="4" t="n"/>
+      <c r="V146" s="4" t="n"/>
     </row>
     <row r="147">
       <c r="A147" s="4" t="n"/>
@@ -3263,6 +3577,7 @@
       <c r="S147" s="4" t="n"/>
       <c r="T147" s="4" t="n"/>
       <c r="U147" s="4" t="n"/>
+      <c r="V147" s="4" t="n"/>
     </row>
     <row r="148">
       <c r="A148" s="4" t="n"/>
@@ -3277,6 +3592,7 @@
       <c r="S148" s="4" t="n"/>
       <c r="T148" s="4" t="n"/>
       <c r="U148" s="4" t="n"/>
+      <c r="V148" s="4" t="n"/>
     </row>
     <row r="149">
       <c r="A149" s="4" t="n"/>
@@ -3291,6 +3607,7 @@
       <c r="S149" s="4" t="n"/>
       <c r="T149" s="4" t="n"/>
       <c r="U149" s="4" t="n"/>
+      <c r="V149" s="4" t="n"/>
     </row>
     <row r="150">
       <c r="A150" s="4" t="n"/>
@@ -3305,6 +3622,7 @@
       <c r="S150" s="4" t="n"/>
       <c r="T150" s="4" t="n"/>
       <c r="U150" s="4" t="n"/>
+      <c r="V150" s="4" t="n"/>
     </row>
     <row r="151">
       <c r="A151" s="4" t="n"/>
@@ -3319,6 +3637,7 @@
       <c r="S151" s="4" t="n"/>
       <c r="T151" s="4" t="n"/>
       <c r="U151" s="4" t="n"/>
+      <c r="V151" s="4" t="n"/>
     </row>
     <row r="152">
       <c r="A152" s="4" t="n"/>
@@ -3333,6 +3652,7 @@
       <c r="S152" s="4" t="n"/>
       <c r="T152" s="4" t="n"/>
       <c r="U152" s="4" t="n"/>
+      <c r="V152" s="4" t="n"/>
     </row>
     <row r="153">
       <c r="A153" s="4" t="n"/>
@@ -3347,6 +3667,7 @@
       <c r="S153" s="4" t="n"/>
       <c r="T153" s="4" t="n"/>
       <c r="U153" s="4" t="n"/>
+      <c r="V153" s="4" t="n"/>
     </row>
     <row r="154">
       <c r="A154" s="4" t="n"/>
@@ -3361,6 +3682,7 @@
       <c r="S154" s="4" t="n"/>
       <c r="T154" s="4" t="n"/>
       <c r="U154" s="4" t="n"/>
+      <c r="V154" s="4" t="n"/>
     </row>
     <row r="155">
       <c r="A155" s="4" t="n"/>
@@ -3375,6 +3697,7 @@
       <c r="S155" s="4" t="n"/>
       <c r="T155" s="4" t="n"/>
       <c r="U155" s="4" t="n"/>
+      <c r="V155" s="4" t="n"/>
     </row>
     <row r="156">
       <c r="A156" s="4" t="n"/>
@@ -3389,6 +3712,7 @@
       <c r="S156" s="4" t="n"/>
       <c r="T156" s="4" t="n"/>
       <c r="U156" s="4" t="n"/>
+      <c r="V156" s="4" t="n"/>
     </row>
     <row r="157">
       <c r="A157" s="4" t="n"/>
@@ -3403,6 +3727,7 @@
       <c r="S157" s="4" t="n"/>
       <c r="T157" s="4" t="n"/>
       <c r="U157" s="4" t="n"/>
+      <c r="V157" s="4" t="n"/>
     </row>
     <row r="158">
       <c r="A158" s="4" t="n"/>
@@ -3417,6 +3742,7 @@
       <c r="S158" s="4" t="n"/>
       <c r="T158" s="4" t="n"/>
       <c r="U158" s="4" t="n"/>
+      <c r="V158" s="4" t="n"/>
     </row>
     <row r="159">
       <c r="A159" s="4" t="n"/>
@@ -3431,6 +3757,7 @@
       <c r="S159" s="4" t="n"/>
       <c r="T159" s="4" t="n"/>
       <c r="U159" s="4" t="n"/>
+      <c r="V159" s="4" t="n"/>
     </row>
     <row r="160">
       <c r="A160" s="4" t="n"/>
@@ -3445,6 +3772,7 @@
       <c r="S160" s="4" t="n"/>
       <c r="T160" s="4" t="n"/>
       <c r="U160" s="4" t="n"/>
+      <c r="V160" s="4" t="n"/>
     </row>
     <row r="161">
       <c r="A161" s="4" t="n"/>
@@ -3459,6 +3787,7 @@
       <c r="S161" s="4" t="n"/>
       <c r="T161" s="4" t="n"/>
       <c r="U161" s="4" t="n"/>
+      <c r="V161" s="4" t="n"/>
     </row>
     <row r="162">
       <c r="A162" s="4" t="n"/>
@@ -3473,6 +3802,7 @@
       <c r="S162" s="4" t="n"/>
       <c r="T162" s="4" t="n"/>
       <c r="U162" s="4" t="n"/>
+      <c r="V162" s="4" t="n"/>
     </row>
     <row r="163">
       <c r="A163" s="4" t="n"/>
@@ -3487,6 +3817,7 @@
       <c r="S163" s="4" t="n"/>
       <c r="T163" s="4" t="n"/>
       <c r="U163" s="4" t="n"/>
+      <c r="V163" s="4" t="n"/>
     </row>
     <row r="164">
       <c r="A164" s="4" t="n"/>
@@ -3501,6 +3832,7 @@
       <c r="S164" s="4" t="n"/>
       <c r="T164" s="4" t="n"/>
       <c r="U164" s="4" t="n"/>
+      <c r="V164" s="4" t="n"/>
     </row>
     <row r="165">
       <c r="A165" s="4" t="n"/>
@@ -3515,6 +3847,7 @@
       <c r="S165" s="4" t="n"/>
       <c r="T165" s="4" t="n"/>
       <c r="U165" s="4" t="n"/>
+      <c r="V165" s="4" t="n"/>
     </row>
     <row r="166">
       <c r="A166" s="4" t="n"/>
@@ -3529,6 +3862,7 @@
       <c r="S166" s="4" t="n"/>
       <c r="T166" s="4" t="n"/>
       <c r="U166" s="4" t="n"/>
+      <c r="V166" s="4" t="n"/>
     </row>
     <row r="167">
       <c r="A167" s="4" t="n"/>
@@ -3543,6 +3877,7 @@
       <c r="S167" s="4" t="n"/>
       <c r="T167" s="4" t="n"/>
       <c r="U167" s="4" t="n"/>
+      <c r="V167" s="4" t="n"/>
     </row>
     <row r="168">
       <c r="A168" s="4" t="n"/>
@@ -3557,6 +3892,7 @@
       <c r="S168" s="4" t="n"/>
       <c r="T168" s="4" t="n"/>
       <c r="U168" s="4" t="n"/>
+      <c r="V168" s="4" t="n"/>
     </row>
     <row r="169">
       <c r="A169" s="4" t="n"/>
@@ -3571,6 +3907,7 @@
       <c r="S169" s="4" t="n"/>
       <c r="T169" s="4" t="n"/>
       <c r="U169" s="4" t="n"/>
+      <c r="V169" s="4" t="n"/>
     </row>
     <row r="170">
       <c r="A170" s="4" t="n"/>
@@ -3585,6 +3922,7 @@
       <c r="S170" s="4" t="n"/>
       <c r="T170" s="4" t="n"/>
       <c r="U170" s="4" t="n"/>
+      <c r="V170" s="4" t="n"/>
     </row>
     <row r="171">
       <c r="A171" s="4" t="n"/>
@@ -3599,6 +3937,7 @@
       <c r="S171" s="4" t="n"/>
       <c r="T171" s="4" t="n"/>
       <c r="U171" s="4" t="n"/>
+      <c r="V171" s="4" t="n"/>
     </row>
     <row r="172">
       <c r="A172" s="4" t="n"/>
@@ -3613,6 +3952,7 @@
       <c r="S172" s="4" t="n"/>
       <c r="T172" s="4" t="n"/>
       <c r="U172" s="4" t="n"/>
+      <c r="V172" s="4" t="n"/>
     </row>
     <row r="173">
       <c r="A173" s="4" t="n"/>
@@ -3627,6 +3967,7 @@
       <c r="S173" s="4" t="n"/>
       <c r="T173" s="4" t="n"/>
       <c r="U173" s="4" t="n"/>
+      <c r="V173" s="4" t="n"/>
     </row>
     <row r="174">
       <c r="A174" s="4" t="n"/>
@@ -3641,6 +3982,7 @@
       <c r="S174" s="4" t="n"/>
       <c r="T174" s="4" t="n"/>
       <c r="U174" s="4" t="n"/>
+      <c r="V174" s="4" t="n"/>
     </row>
     <row r="175">
       <c r="A175" s="4" t="n"/>
@@ -3655,6 +3997,7 @@
       <c r="S175" s="4" t="n"/>
       <c r="T175" s="4" t="n"/>
       <c r="U175" s="4" t="n"/>
+      <c r="V175" s="4" t="n"/>
     </row>
     <row r="176">
       <c r="A176" s="4" t="n"/>
@@ -3669,6 +4012,7 @@
       <c r="S176" s="4" t="n"/>
       <c r="T176" s="4" t="n"/>
       <c r="U176" s="4" t="n"/>
+      <c r="V176" s="4" t="n"/>
     </row>
     <row r="177">
       <c r="A177" s="4" t="n"/>
@@ -3683,6 +4027,7 @@
       <c r="S177" s="4" t="n"/>
       <c r="T177" s="4" t="n"/>
       <c r="U177" s="4" t="n"/>
+      <c r="V177" s="4" t="n"/>
     </row>
     <row r="178">
       <c r="A178" s="4" t="n"/>
@@ -3697,6 +4042,7 @@
       <c r="S178" s="4" t="n"/>
       <c r="T178" s="4" t="n"/>
       <c r="U178" s="4" t="n"/>
+      <c r="V178" s="4" t="n"/>
     </row>
     <row r="179">
       <c r="A179" s="4" t="n"/>
@@ -3711,6 +4057,7 @@
       <c r="S179" s="4" t="n"/>
       <c r="T179" s="4" t="n"/>
       <c r="U179" s="4" t="n"/>
+      <c r="V179" s="4" t="n"/>
     </row>
     <row r="180">
       <c r="A180" s="4" t="n"/>
@@ -3725,6 +4072,7 @@
       <c r="S180" s="4" t="n"/>
       <c r="T180" s="4" t="n"/>
       <c r="U180" s="4" t="n"/>
+      <c r="V180" s="4" t="n"/>
     </row>
     <row r="181">
       <c r="A181" s="4" t="n"/>
@@ -3739,6 +4087,7 @@
       <c r="S181" s="4" t="n"/>
       <c r="T181" s="4" t="n"/>
       <c r="U181" s="4" t="n"/>
+      <c r="V181" s="4" t="n"/>
     </row>
     <row r="182">
       <c r="A182" s="4" t="n"/>
@@ -3753,6 +4102,7 @@
       <c r="S182" s="4" t="n"/>
       <c r="T182" s="4" t="n"/>
       <c r="U182" s="4" t="n"/>
+      <c r="V182" s="4" t="n"/>
     </row>
     <row r="183">
       <c r="A183" s="4" t="n"/>
@@ -3767,6 +4117,7 @@
       <c r="S183" s="4" t="n"/>
       <c r="T183" s="4" t="n"/>
       <c r="U183" s="4" t="n"/>
+      <c r="V183" s="4" t="n"/>
     </row>
     <row r="184">
       <c r="A184" s="4" t="n"/>
@@ -3781,6 +4132,7 @@
       <c r="S184" s="4" t="n"/>
       <c r="T184" s="4" t="n"/>
       <c r="U184" s="4" t="n"/>
+      <c r="V184" s="4" t="n"/>
     </row>
     <row r="185">
       <c r="A185" s="4" t="n"/>
@@ -3795,6 +4147,7 @@
       <c r="S185" s="4" t="n"/>
       <c r="T185" s="4" t="n"/>
       <c r="U185" s="4" t="n"/>
+      <c r="V185" s="4" t="n"/>
     </row>
     <row r="186">
       <c r="A186" s="4" t="n"/>
@@ -3809,6 +4162,7 @@
       <c r="S186" s="4" t="n"/>
       <c r="T186" s="4" t="n"/>
       <c r="U186" s="4" t="n"/>
+      <c r="V186" s="4" t="n"/>
     </row>
     <row r="187">
       <c r="A187" s="4" t="n"/>
@@ -3823,6 +4177,7 @@
       <c r="S187" s="4" t="n"/>
       <c r="T187" s="4" t="n"/>
       <c r="U187" s="4" t="n"/>
+      <c r="V187" s="4" t="n"/>
     </row>
     <row r="188">
       <c r="A188" s="4" t="n"/>
@@ -3837,6 +4192,7 @@
       <c r="S188" s="4" t="n"/>
       <c r="T188" s="4" t="n"/>
       <c r="U188" s="4" t="n"/>
+      <c r="V188" s="4" t="n"/>
     </row>
     <row r="189">
       <c r="A189" s="4" t="n"/>
@@ -3851,6 +4207,7 @@
       <c r="S189" s="4" t="n"/>
       <c r="T189" s="4" t="n"/>
       <c r="U189" s="4" t="n"/>
+      <c r="V189" s="4" t="n"/>
     </row>
     <row r="190">
       <c r="A190" s="4" t="n"/>
@@ -3865,6 +4222,7 @@
       <c r="S190" s="4" t="n"/>
       <c r="T190" s="4" t="n"/>
       <c r="U190" s="4" t="n"/>
+      <c r="V190" s="4" t="n"/>
     </row>
     <row r="191">
       <c r="A191" s="4" t="n"/>
@@ -3879,6 +4237,7 @@
       <c r="S191" s="4" t="n"/>
       <c r="T191" s="4" t="n"/>
       <c r="U191" s="4" t="n"/>
+      <c r="V191" s="4" t="n"/>
     </row>
     <row r="192">
       <c r="A192" s="4" t="n"/>
@@ -3893,6 +4252,7 @@
       <c r="S192" s="4" t="n"/>
       <c r="T192" s="4" t="n"/>
       <c r="U192" s="4" t="n"/>
+      <c r="V192" s="4" t="n"/>
     </row>
     <row r="193">
       <c r="A193" s="4" t="n"/>
@@ -3907,6 +4267,7 @@
       <c r="S193" s="4" t="n"/>
       <c r="T193" s="4" t="n"/>
       <c r="U193" s="4" t="n"/>
+      <c r="V193" s="4" t="n"/>
     </row>
     <row r="194">
       <c r="A194" s="4" t="n"/>
@@ -3921,6 +4282,7 @@
       <c r="S194" s="4" t="n"/>
       <c r="T194" s="4" t="n"/>
       <c r="U194" s="4" t="n"/>
+      <c r="V194" s="4" t="n"/>
     </row>
     <row r="195">
       <c r="A195" s="4" t="n"/>
@@ -3935,6 +4297,7 @@
       <c r="S195" s="4" t="n"/>
       <c r="T195" s="4" t="n"/>
       <c r="U195" s="4" t="n"/>
+      <c r="V195" s="4" t="n"/>
     </row>
     <row r="196">
       <c r="A196" s="4" t="n"/>
@@ -3949,6 +4312,7 @@
       <c r="S196" s="4" t="n"/>
       <c r="T196" s="4" t="n"/>
       <c r="U196" s="4" t="n"/>
+      <c r="V196" s="4" t="n"/>
     </row>
     <row r="197">
       <c r="A197" s="4" t="n"/>
@@ -3963,6 +4327,7 @@
       <c r="S197" s="4" t="n"/>
       <c r="T197" s="4" t="n"/>
       <c r="U197" s="4" t="n"/>
+      <c r="V197" s="4" t="n"/>
     </row>
     <row r="198">
       <c r="A198" s="4" t="n"/>
@@ -3977,6 +4342,7 @@
       <c r="S198" s="4" t="n"/>
       <c r="T198" s="4" t="n"/>
       <c r="U198" s="4" t="n"/>
+      <c r="V198" s="4" t="n"/>
     </row>
     <row r="199">
       <c r="A199" s="4" t="n"/>
@@ -3991,6 +4357,7 @@
       <c r="S199" s="4" t="n"/>
       <c r="T199" s="4" t="n"/>
       <c r="U199" s="4" t="n"/>
+      <c r="V199" s="4" t="n"/>
     </row>
     <row r="200">
       <c r="A200" s="4" t="n"/>
@@ -4005,6 +4372,7 @@
       <c r="S200" s="4" t="n"/>
       <c r="T200" s="4" t="n"/>
       <c r="U200" s="4" t="n"/>
+      <c r="V200" s="4" t="n"/>
     </row>
     <row r="201">
       <c r="A201" s="4" t="n"/>
@@ -4019,6 +4387,7 @@
       <c r="S201" s="4" t="n"/>
       <c r="T201" s="4" t="n"/>
       <c r="U201" s="4" t="n"/>
+      <c r="V201" s="4" t="n"/>
     </row>
     <row r="202">
       <c r="A202" s="4" t="n"/>
@@ -4033,6 +4402,7 @@
       <c r="S202" s="4" t="n"/>
       <c r="T202" s="4" t="n"/>
       <c r="U202" s="4" t="n"/>
+      <c r="V202" s="4" t="n"/>
     </row>
     <row r="203">
       <c r="A203" s="4" t="n"/>
@@ -4047,6 +4417,7 @@
       <c r="S203" s="4" t="n"/>
       <c r="T203" s="4" t="n"/>
       <c r="U203" s="4" t="n"/>
+      <c r="V203" s="4" t="n"/>
     </row>
     <row r="204">
       <c r="A204" s="4" t="n"/>
@@ -4061,6 +4432,7 @@
       <c r="S204" s="4" t="n"/>
       <c r="T204" s="4" t="n"/>
       <c r="U204" s="4" t="n"/>
+      <c r="V204" s="4" t="n"/>
     </row>
     <row r="205">
       <c r="A205" s="4" t="n"/>
@@ -4075,6 +4447,7 @@
       <c r="S205" s="4" t="n"/>
       <c r="T205" s="4" t="n"/>
       <c r="U205" s="4" t="n"/>
+      <c r="V205" s="4" t="n"/>
     </row>
     <row r="206">
       <c r="A206" s="4" t="n"/>
@@ -4089,6 +4462,7 @@
       <c r="S206" s="4" t="n"/>
       <c r="T206" s="4" t="n"/>
       <c r="U206" s="4" t="n"/>
+      <c r="V206" s="4" t="n"/>
     </row>
     <row r="207">
       <c r="A207" s="4" t="n"/>
@@ -4103,6 +4477,7 @@
       <c r="S207" s="4" t="n"/>
       <c r="T207" s="4" t="n"/>
       <c r="U207" s="4" t="n"/>
+      <c r="V207" s="4" t="n"/>
     </row>
     <row r="208">
       <c r="A208" s="4" t="n"/>
@@ -4117,6 +4492,7 @@
       <c r="S208" s="4" t="n"/>
       <c r="T208" s="4" t="n"/>
       <c r="U208" s="4" t="n"/>
+      <c r="V208" s="4" t="n"/>
     </row>
     <row r="209">
       <c r="A209" s="4" t="n"/>
@@ -4131,6 +4507,7 @@
       <c r="S209" s="4" t="n"/>
       <c r="T209" s="4" t="n"/>
       <c r="U209" s="4" t="n"/>
+      <c r="V209" s="4" t="n"/>
     </row>
     <row r="210">
       <c r="A210" s="4" t="n"/>
@@ -4145,6 +4522,7 @@
       <c r="S210" s="4" t="n"/>
       <c r="T210" s="4" t="n"/>
       <c r="U210" s="4" t="n"/>
+      <c r="V210" s="4" t="n"/>
     </row>
     <row r="211">
       <c r="A211" s="4" t="n"/>
@@ -4159,6 +4537,7 @@
       <c r="S211" s="4" t="n"/>
       <c r="T211" s="4" t="n"/>
       <c r="U211" s="4" t="n"/>
+      <c r="V211" s="4" t="n"/>
     </row>
     <row r="212">
       <c r="A212" s="4" t="n"/>
@@ -4173,6 +4552,7 @@
       <c r="S212" s="4" t="n"/>
       <c r="T212" s="4" t="n"/>
       <c r="U212" s="4" t="n"/>
+      <c r="V212" s="4" t="n"/>
     </row>
     <row r="213">
       <c r="A213" s="4" t="n"/>
@@ -4187,6 +4567,7 @@
       <c r="S213" s="4" t="n"/>
       <c r="T213" s="4" t="n"/>
       <c r="U213" s="4" t="n"/>
+      <c r="V213" s="4" t="n"/>
     </row>
     <row r="214">
       <c r="A214" s="4" t="n"/>
@@ -4201,6 +4582,7 @@
       <c r="S214" s="4" t="n"/>
       <c r="T214" s="4" t="n"/>
       <c r="U214" s="4" t="n"/>
+      <c r="V214" s="4" t="n"/>
     </row>
     <row r="215">
       <c r="A215" s="4" t="n"/>
@@ -4215,6 +4597,7 @@
       <c r="S215" s="4" t="n"/>
       <c r="T215" s="4" t="n"/>
       <c r="U215" s="4" t="n"/>
+      <c r="V215" s="4" t="n"/>
     </row>
     <row r="216">
       <c r="A216" s="4" t="n"/>
@@ -4229,6 +4612,7 @@
       <c r="S216" s="4" t="n"/>
       <c r="T216" s="4" t="n"/>
       <c r="U216" s="4" t="n"/>
+      <c r="V216" s="4" t="n"/>
     </row>
     <row r="217">
       <c r="A217" s="4" t="n"/>
@@ -4243,6 +4627,7 @@
       <c r="S217" s="4" t="n"/>
       <c r="T217" s="4" t="n"/>
       <c r="U217" s="4" t="n"/>
+      <c r="V217" s="4" t="n"/>
     </row>
     <row r="218">
       <c r="A218" s="4" t="n"/>
@@ -4257,6 +4642,7 @@
       <c r="S218" s="4" t="n"/>
       <c r="T218" s="4" t="n"/>
       <c r="U218" s="4" t="n"/>
+      <c r="V218" s="4" t="n"/>
     </row>
     <row r="219">
       <c r="A219" s="4" t="n"/>
@@ -4271,6 +4657,7 @@
       <c r="S219" s="4" t="n"/>
       <c r="T219" s="4" t="n"/>
       <c r="U219" s="4" t="n"/>
+      <c r="V219" s="4" t="n"/>
     </row>
     <row r="220">
       <c r="A220" s="4" t="n"/>
@@ -4285,6 +4672,7 @@
       <c r="S220" s="4" t="n"/>
       <c r="T220" s="4" t="n"/>
       <c r="U220" s="4" t="n"/>
+      <c r="V220" s="4" t="n"/>
     </row>
     <row r="221">
       <c r="A221" s="4" t="n"/>
@@ -4299,6 +4687,7 @@
       <c r="S221" s="4" t="n"/>
       <c r="T221" s="4" t="n"/>
       <c r="U221" s="4" t="n"/>
+      <c r="V221" s="4" t="n"/>
     </row>
     <row r="222">
       <c r="A222" s="4" t="n"/>
@@ -4313,6 +4702,7 @@
       <c r="S222" s="4" t="n"/>
       <c r="T222" s="4" t="n"/>
       <c r="U222" s="4" t="n"/>
+      <c r="V222" s="4" t="n"/>
     </row>
     <row r="223">
       <c r="A223" s="4" t="n"/>
@@ -4327,6 +4717,7 @@
       <c r="S223" s="4" t="n"/>
       <c r="T223" s="4" t="n"/>
       <c r="U223" s="4" t="n"/>
+      <c r="V223" s="4" t="n"/>
     </row>
     <row r="224">
       <c r="A224" s="4" t="n"/>
@@ -4341,6 +4732,7 @@
       <c r="S224" s="4" t="n"/>
       <c r="T224" s="4" t="n"/>
       <c r="U224" s="4" t="n"/>
+      <c r="V224" s="4" t="n"/>
     </row>
     <row r="225">
       <c r="A225" s="4" t="n"/>
@@ -4355,6 +4747,7 @@
       <c r="S225" s="4" t="n"/>
       <c r="T225" s="4" t="n"/>
       <c r="U225" s="4" t="n"/>
+      <c r="V225" s="4" t="n"/>
     </row>
     <row r="226">
       <c r="A226" s="4" t="n"/>
@@ -4369,6 +4762,7 @@
       <c r="S226" s="4" t="n"/>
       <c r="T226" s="4" t="n"/>
       <c r="U226" s="4" t="n"/>
+      <c r="V226" s="4" t="n"/>
     </row>
     <row r="227">
       <c r="A227" s="4" t="n"/>
@@ -4383,6 +4777,7 @@
       <c r="S227" s="4" t="n"/>
       <c r="T227" s="4" t="n"/>
       <c r="U227" s="4" t="n"/>
+      <c r="V227" s="4" t="n"/>
     </row>
     <row r="228">
       <c r="A228" s="4" t="n"/>
@@ -4397,6 +4792,7 @@
       <c r="S228" s="4" t="n"/>
       <c r="T228" s="4" t="n"/>
       <c r="U228" s="4" t="n"/>
+      <c r="V228" s="4" t="n"/>
     </row>
     <row r="229">
       <c r="A229" s="4" t="n"/>
@@ -4411,6 +4807,7 @@
       <c r="S229" s="4" t="n"/>
       <c r="T229" s="4" t="n"/>
       <c r="U229" s="4" t="n"/>
+      <c r="V229" s="4" t="n"/>
     </row>
     <row r="230">
       <c r="A230" s="4" t="n"/>
@@ -4425,6 +4822,7 @@
       <c r="S230" s="4" t="n"/>
       <c r="T230" s="4" t="n"/>
       <c r="U230" s="4" t="n"/>
+      <c r="V230" s="4" t="n"/>
     </row>
     <row r="231">
       <c r="A231" s="4" t="n"/>
@@ -4439,6 +4837,7 @@
       <c r="S231" s="4" t="n"/>
       <c r="T231" s="4" t="n"/>
       <c r="U231" s="4" t="n"/>
+      <c r="V231" s="4" t="n"/>
     </row>
     <row r="232">
       <c r="A232" s="4" t="n"/>
@@ -4453,6 +4852,7 @@
       <c r="S232" s="4" t="n"/>
       <c r="T232" s="4" t="n"/>
       <c r="U232" s="4" t="n"/>
+      <c r="V232" s="4" t="n"/>
     </row>
     <row r="233">
       <c r="A233" s="4" t="n"/>
@@ -4467,6 +4867,7 @@
       <c r="S233" s="4" t="n"/>
       <c r="T233" s="4" t="n"/>
       <c r="U233" s="4" t="n"/>
+      <c r="V233" s="4" t="n"/>
     </row>
     <row r="234">
       <c r="A234" s="4" t="n"/>
@@ -4481,6 +4882,7 @@
       <c r="S234" s="4" t="n"/>
       <c r="T234" s="4" t="n"/>
       <c r="U234" s="4" t="n"/>
+      <c r="V234" s="4" t="n"/>
     </row>
     <row r="235">
       <c r="A235" s="4" t="n"/>
@@ -4495,6 +4897,7 @@
       <c r="S235" s="4" t="n"/>
       <c r="T235" s="4" t="n"/>
       <c r="U235" s="4" t="n"/>
+      <c r="V235" s="4" t="n"/>
     </row>
     <row r="236">
       <c r="A236" s="4" t="n"/>
@@ -4509,6 +4912,7 @@
       <c r="S236" s="4" t="n"/>
       <c r="T236" s="4" t="n"/>
       <c r="U236" s="4" t="n"/>
+      <c r="V236" s="4" t="n"/>
     </row>
     <row r="237">
       <c r="A237" s="4" t="n"/>
@@ -4523,6 +4927,7 @@
       <c r="S237" s="4" t="n"/>
       <c r="T237" s="4" t="n"/>
       <c r="U237" s="4" t="n"/>
+      <c r="V237" s="4" t="n"/>
     </row>
     <row r="238">
       <c r="A238" s="4" t="n"/>
@@ -4537,6 +4942,7 @@
       <c r="S238" s="4" t="n"/>
       <c r="T238" s="4" t="n"/>
       <c r="U238" s="4" t="n"/>
+      <c r="V238" s="4" t="n"/>
     </row>
     <row r="239">
       <c r="A239" s="4" t="n"/>
@@ -4551,6 +4957,7 @@
       <c r="S239" s="4" t="n"/>
       <c r="T239" s="4" t="n"/>
       <c r="U239" s="4" t="n"/>
+      <c r="V239" s="4" t="n"/>
     </row>
     <row r="240">
       <c r="A240" s="4" t="n"/>
@@ -4565,6 +4972,7 @@
       <c r="S240" s="4" t="n"/>
       <c r="T240" s="4" t="n"/>
       <c r="U240" s="4" t="n"/>
+      <c r="V240" s="4" t="n"/>
     </row>
     <row r="241">
       <c r="A241" s="4" t="n"/>
@@ -4579,6 +4987,7 @@
       <c r="S241" s="4" t="n"/>
       <c r="T241" s="4" t="n"/>
       <c r="U241" s="4" t="n"/>
+      <c r="V241" s="4" t="n"/>
     </row>
     <row r="242">
       <c r="A242" s="4" t="n"/>
@@ -4593,6 +5002,7 @@
       <c r="S242" s="4" t="n"/>
       <c r="T242" s="4" t="n"/>
       <c r="U242" s="4" t="n"/>
+      <c r="V242" s="4" t="n"/>
     </row>
     <row r="243">
       <c r="A243" s="4" t="n"/>
@@ -4607,6 +5017,7 @@
       <c r="S243" s="4" t="n"/>
       <c r="T243" s="4" t="n"/>
       <c r="U243" s="4" t="n"/>
+      <c r="V243" s="4" t="n"/>
     </row>
     <row r="244">
       <c r="A244" s="4" t="n"/>
@@ -4621,6 +5032,7 @@
       <c r="S244" s="4" t="n"/>
       <c r="T244" s="4" t="n"/>
       <c r="U244" s="4" t="n"/>
+      <c r="V244" s="4" t="n"/>
     </row>
     <row r="245">
       <c r="A245" s="4" t="n"/>
@@ -4635,6 +5047,7 @@
       <c r="S245" s="4" t="n"/>
       <c r="T245" s="4" t="n"/>
       <c r="U245" s="4" t="n"/>
+      <c r="V245" s="4" t="n"/>
     </row>
     <row r="246">
       <c r="A246" s="4" t="n"/>
@@ -4649,6 +5062,7 @@
       <c r="S246" s="4" t="n"/>
       <c r="T246" s="4" t="n"/>
       <c r="U246" s="4" t="n"/>
+      <c r="V246" s="4" t="n"/>
     </row>
     <row r="247">
       <c r="A247" s="4" t="n"/>
@@ -4663,6 +5077,7 @@
       <c r="S247" s="4" t="n"/>
       <c r="T247" s="4" t="n"/>
       <c r="U247" s="4" t="n"/>
+      <c r="V247" s="4" t="n"/>
     </row>
     <row r="248">
       <c r="A248" s="4" t="n"/>
@@ -4677,6 +5092,7 @@
       <c r="S248" s="4" t="n"/>
       <c r="T248" s="4" t="n"/>
       <c r="U248" s="4" t="n"/>
+      <c r="V248" s="4" t="n"/>
     </row>
     <row r="249">
       <c r="A249" s="4" t="n"/>
@@ -4691,6 +5107,7 @@
       <c r="S249" s="4" t="n"/>
       <c r="T249" s="4" t="n"/>
       <c r="U249" s="4" t="n"/>
+      <c r="V249" s="4" t="n"/>
     </row>
     <row r="250">
       <c r="A250" s="4" t="n"/>
@@ -4705,6 +5122,7 @@
       <c r="S250" s="4" t="n"/>
       <c r="T250" s="4" t="n"/>
       <c r="U250" s="4" t="n"/>
+      <c r="V250" s="4" t="n"/>
     </row>
     <row r="251">
       <c r="A251" s="4" t="n"/>
@@ -4719,6 +5137,7 @@
       <c r="S251" s="4" t="n"/>
       <c r="T251" s="4" t="n"/>
       <c r="U251" s="4" t="n"/>
+      <c r="V251" s="4" t="n"/>
     </row>
     <row r="252">
       <c r="A252" s="4" t="n"/>
@@ -4733,6 +5152,7 @@
       <c r="S252" s="4" t="n"/>
       <c r="T252" s="4" t="n"/>
       <c r="U252" s="4" t="n"/>
+      <c r="V252" s="4" t="n"/>
     </row>
     <row r="253">
       <c r="A253" s="4" t="n"/>
@@ -4747,6 +5167,7 @@
       <c r="S253" s="4" t="n"/>
       <c r="T253" s="4" t="n"/>
       <c r="U253" s="4" t="n"/>
+      <c r="V253" s="4" t="n"/>
     </row>
     <row r="254">
       <c r="A254" s="4" t="n"/>
@@ -4761,6 +5182,7 @@
       <c r="S254" s="4" t="n"/>
       <c r="T254" s="4" t="n"/>
       <c r="U254" s="4" t="n"/>
+      <c r="V254" s="4" t="n"/>
     </row>
     <row r="255">
       <c r="A255" s="4" t="n"/>
@@ -4775,6 +5197,7 @@
       <c r="S255" s="4" t="n"/>
       <c r="T255" s="4" t="n"/>
       <c r="U255" s="4" t="n"/>
+      <c r="V255" s="4" t="n"/>
     </row>
     <row r="256">
       <c r="A256" s="4" t="n"/>
@@ -4789,6 +5212,7 @@
       <c r="S256" s="4" t="n"/>
       <c r="T256" s="4" t="n"/>
       <c r="U256" s="4" t="n"/>
+      <c r="V256" s="4" t="n"/>
     </row>
     <row r="257">
       <c r="A257" s="4" t="n"/>
@@ -4803,6 +5227,7 @@
       <c r="S257" s="4" t="n"/>
       <c r="T257" s="4" t="n"/>
       <c r="U257" s="4" t="n"/>
+      <c r="V257" s="4" t="n"/>
     </row>
     <row r="258">
       <c r="A258" s="4" t="n"/>
@@ -4817,6 +5242,7 @@
       <c r="S258" s="4" t="n"/>
       <c r="T258" s="4" t="n"/>
       <c r="U258" s="4" t="n"/>
+      <c r="V258" s="4" t="n"/>
     </row>
     <row r="259">
       <c r="A259" s="4" t="n"/>
@@ -4831,6 +5257,7 @@
       <c r="S259" s="4" t="n"/>
       <c r="T259" s="4" t="n"/>
       <c r="U259" s="4" t="n"/>
+      <c r="V259" s="4" t="n"/>
     </row>
     <row r="260">
       <c r="A260" s="4" t="n"/>
@@ -4845,6 +5272,7 @@
       <c r="S260" s="4" t="n"/>
       <c r="T260" s="4" t="n"/>
       <c r="U260" s="4" t="n"/>
+      <c r="V260" s="4" t="n"/>
     </row>
     <row r="261">
       <c r="A261" s="4" t="n"/>
@@ -4859,6 +5287,7 @@
       <c r="S261" s="4" t="n"/>
       <c r="T261" s="4" t="n"/>
       <c r="U261" s="4" t="n"/>
+      <c r="V261" s="4" t="n"/>
     </row>
     <row r="262">
       <c r="A262" s="4" t="n"/>
@@ -4873,6 +5302,7 @@
       <c r="S262" s="4" t="n"/>
       <c r="T262" s="4" t="n"/>
       <c r="U262" s="4" t="n"/>
+      <c r="V262" s="4" t="n"/>
     </row>
     <row r="263">
       <c r="A263" s="4" t="n"/>
@@ -4887,6 +5317,7 @@
       <c r="S263" s="4" t="n"/>
       <c r="T263" s="4" t="n"/>
       <c r="U263" s="4" t="n"/>
+      <c r="V263" s="4" t="n"/>
     </row>
     <row r="264">
       <c r="A264" s="4" t="n"/>
@@ -4901,6 +5332,7 @@
       <c r="S264" s="4" t="n"/>
       <c r="T264" s="4" t="n"/>
       <c r="U264" s="4" t="n"/>
+      <c r="V264" s="4" t="n"/>
     </row>
     <row r="265">
       <c r="A265" s="4" t="n"/>
@@ -4915,6 +5347,7 @@
       <c r="S265" s="4" t="n"/>
       <c r="T265" s="4" t="n"/>
       <c r="U265" s="4" t="n"/>
+      <c r="V265" s="4" t="n"/>
     </row>
     <row r="266">
       <c r="A266" s="4" t="n"/>
@@ -4929,6 +5362,7 @@
       <c r="S266" s="4" t="n"/>
       <c r="T266" s="4" t="n"/>
       <c r="U266" s="4" t="n"/>
+      <c r="V266" s="4" t="n"/>
     </row>
     <row r="267">
       <c r="A267" s="4" t="n"/>
@@ -4943,6 +5377,7 @@
       <c r="S267" s="4" t="n"/>
       <c r="T267" s="4" t="n"/>
       <c r="U267" s="4" t="n"/>
+      <c r="V267" s="4" t="n"/>
     </row>
     <row r="268">
       <c r="A268" s="4" t="n"/>
@@ -4957,6 +5392,7 @@
       <c r="S268" s="4" t="n"/>
       <c r="T268" s="4" t="n"/>
       <c r="U268" s="4" t="n"/>
+      <c r="V268" s="4" t="n"/>
     </row>
     <row r="269">
       <c r="A269" s="4" t="n"/>
@@ -4971,6 +5407,7 @@
       <c r="S269" s="4" t="n"/>
       <c r="T269" s="4" t="n"/>
       <c r="U269" s="4" t="n"/>
+      <c r="V269" s="4" t="n"/>
     </row>
     <row r="270">
       <c r="A270" s="4" t="n"/>
@@ -4985,6 +5422,7 @@
       <c r="S270" s="4" t="n"/>
       <c r="T270" s="4" t="n"/>
       <c r="U270" s="4" t="n"/>
+      <c r="V270" s="4" t="n"/>
     </row>
     <row r="271">
       <c r="A271" s="4" t="n"/>
@@ -4999,6 +5437,7 @@
       <c r="S271" s="4" t="n"/>
       <c r="T271" s="4" t="n"/>
       <c r="U271" s="4" t="n"/>
+      <c r="V271" s="4" t="n"/>
     </row>
     <row r="272">
       <c r="A272" s="4" t="n"/>
@@ -5013,6 +5452,7 @@
       <c r="S272" s="4" t="n"/>
       <c r="T272" s="4" t="n"/>
       <c r="U272" s="4" t="n"/>
+      <c r="V272" s="4" t="n"/>
     </row>
     <row r="273">
       <c r="A273" s="4" t="n"/>
@@ -5027,6 +5467,7 @@
       <c r="S273" s="4" t="n"/>
       <c r="T273" s="4" t="n"/>
       <c r="U273" s="4" t="n"/>
+      <c r="V273" s="4" t="n"/>
     </row>
     <row r="274">
       <c r="A274" s="4" t="n"/>
@@ -5041,6 +5482,7 @@
       <c r="S274" s="4" t="n"/>
       <c r="T274" s="4" t="n"/>
       <c r="U274" s="4" t="n"/>
+      <c r="V274" s="4" t="n"/>
     </row>
     <row r="275">
       <c r="A275" s="4" t="n"/>
@@ -5055,6 +5497,7 @@
       <c r="S275" s="4" t="n"/>
       <c r="T275" s="4" t="n"/>
       <c r="U275" s="4" t="n"/>
+      <c r="V275" s="4" t="n"/>
     </row>
     <row r="276">
       <c r="A276" s="4" t="n"/>
@@ -5069,6 +5512,7 @@
       <c r="S276" s="4" t="n"/>
       <c r="T276" s="4" t="n"/>
       <c r="U276" s="4" t="n"/>
+      <c r="V276" s="4" t="n"/>
     </row>
     <row r="277">
       <c r="A277" s="4" t="n"/>
@@ -5083,6 +5527,7 @@
       <c r="S277" s="4" t="n"/>
       <c r="T277" s="4" t="n"/>
       <c r="U277" s="4" t="n"/>
+      <c r="V277" s="4" t="n"/>
     </row>
     <row r="278">
       <c r="A278" s="4" t="n"/>
@@ -5097,6 +5542,7 @@
       <c r="S278" s="4" t="n"/>
       <c r="T278" s="4" t="n"/>
       <c r="U278" s="4" t="n"/>
+      <c r="V278" s="4" t="n"/>
     </row>
     <row r="279">
       <c r="A279" s="4" t="n"/>
@@ -5111,6 +5557,7 @@
       <c r="S279" s="4" t="n"/>
       <c r="T279" s="4" t="n"/>
       <c r="U279" s="4" t="n"/>
+      <c r="V279" s="4" t="n"/>
     </row>
     <row r="280">
       <c r="A280" s="4" t="n"/>
@@ -5125,6 +5572,7 @@
       <c r="S280" s="4" t="n"/>
       <c r="T280" s="4" t="n"/>
       <c r="U280" s="4" t="n"/>
+      <c r="V280" s="4" t="n"/>
     </row>
     <row r="281">
       <c r="A281" s="4" t="n"/>
@@ -5139,6 +5587,7 @@
       <c r="S281" s="4" t="n"/>
       <c r="T281" s="4" t="n"/>
       <c r="U281" s="4" t="n"/>
+      <c r="V281" s="4" t="n"/>
     </row>
     <row r="282">
       <c r="A282" s="4" t="n"/>
@@ -5153,6 +5602,7 @@
       <c r="S282" s="4" t="n"/>
       <c r="T282" s="4" t="n"/>
       <c r="U282" s="4" t="n"/>
+      <c r="V282" s="4" t="n"/>
     </row>
     <row r="283">
       <c r="A283" s="4" t="n"/>
@@ -5167,6 +5617,7 @@
       <c r="S283" s="4" t="n"/>
       <c r="T283" s="4" t="n"/>
       <c r="U283" s="4" t="n"/>
+      <c r="V283" s="4" t="n"/>
     </row>
     <row r="284">
       <c r="A284" s="4" t="n"/>
@@ -5181,6 +5632,7 @@
       <c r="S284" s="4" t="n"/>
       <c r="T284" s="4" t="n"/>
       <c r="U284" s="4" t="n"/>
+      <c r="V284" s="4" t="n"/>
     </row>
     <row r="285">
       <c r="A285" s="4" t="n"/>
@@ -5195,6 +5647,7 @@
       <c r="S285" s="4" t="n"/>
       <c r="T285" s="4" t="n"/>
       <c r="U285" s="4" t="n"/>
+      <c r="V285" s="4" t="n"/>
     </row>
     <row r="286">
       <c r="A286" s="4" t="n"/>
@@ -5209,6 +5662,7 @@
       <c r="S286" s="4" t="n"/>
       <c r="T286" s="4" t="n"/>
       <c r="U286" s="4" t="n"/>
+      <c r="V286" s="4" t="n"/>
     </row>
     <row r="287">
       <c r="A287" s="4" t="n"/>
@@ -5223,6 +5677,7 @@
       <c r="S287" s="4" t="n"/>
       <c r="T287" s="4" t="n"/>
       <c r="U287" s="4" t="n"/>
+      <c r="V287" s="4" t="n"/>
     </row>
     <row r="288">
       <c r="A288" s="4" t="n"/>
@@ -5237,6 +5692,7 @@
       <c r="S288" s="4" t="n"/>
       <c r="T288" s="4" t="n"/>
       <c r="U288" s="4" t="n"/>
+      <c r="V288" s="4" t="n"/>
     </row>
     <row r="289">
       <c r="A289" s="4" t="n"/>
@@ -5251,6 +5707,7 @@
       <c r="S289" s="4" t="n"/>
       <c r="T289" s="4" t="n"/>
       <c r="U289" s="4" t="n"/>
+      <c r="V289" s="4" t="n"/>
     </row>
     <row r="290">
       <c r="A290" s="4" t="n"/>
@@ -5265,6 +5722,7 @@
       <c r="S290" s="4" t="n"/>
       <c r="T290" s="4" t="n"/>
       <c r="U290" s="4" t="n"/>
+      <c r="V290" s="4" t="n"/>
     </row>
     <row r="291">
       <c r="A291" s="4" t="n"/>
@@ -5279,6 +5737,7 @@
       <c r="S291" s="4" t="n"/>
       <c r="T291" s="4" t="n"/>
       <c r="U291" s="4" t="n"/>
+      <c r="V291" s="4" t="n"/>
     </row>
     <row r="292">
       <c r="A292" s="4" t="n"/>
@@ -5293,6 +5752,7 @@
       <c r="S292" s="4" t="n"/>
       <c r="T292" s="4" t="n"/>
       <c r="U292" s="4" t="n"/>
+      <c r="V292" s="4" t="n"/>
     </row>
     <row r="293">
       <c r="A293" s="4" t="n"/>
@@ -5307,6 +5767,7 @@
       <c r="S293" s="4" t="n"/>
       <c r="T293" s="4" t="n"/>
       <c r="U293" s="4" t="n"/>
+      <c r="V293" s="4" t="n"/>
     </row>
     <row r="294">
       <c r="A294" s="4" t="n"/>
@@ -5321,6 +5782,7 @@
       <c r="S294" s="4" t="n"/>
       <c r="T294" s="4" t="n"/>
       <c r="U294" s="4" t="n"/>
+      <c r="V294" s="4" t="n"/>
     </row>
     <row r="295">
       <c r="A295" s="4" t="n"/>
@@ -5335,6 +5797,7 @@
       <c r="S295" s="4" t="n"/>
       <c r="T295" s="4" t="n"/>
       <c r="U295" s="4" t="n"/>
+      <c r="V295" s="4" t="n"/>
     </row>
     <row r="296">
       <c r="A296" s="4" t="n"/>
@@ -5349,6 +5812,7 @@
       <c r="S296" s="4" t="n"/>
       <c r="T296" s="4" t="n"/>
       <c r="U296" s="4" t="n"/>
+      <c r="V296" s="4" t="n"/>
     </row>
     <row r="297">
       <c r="A297" s="4" t="n"/>
@@ -5363,6 +5827,7 @@
       <c r="S297" s="4" t="n"/>
       <c r="T297" s="4" t="n"/>
       <c r="U297" s="4" t="n"/>
+      <c r="V297" s="4" t="n"/>
     </row>
     <row r="298">
       <c r="A298" s="4" t="n"/>
@@ -5377,6 +5842,7 @@
       <c r="S298" s="4" t="n"/>
       <c r="T298" s="4" t="n"/>
       <c r="U298" s="4" t="n"/>
+      <c r="V298" s="4" t="n"/>
     </row>
     <row r="299">
       <c r="A299" s="4" t="n"/>
@@ -5391,6 +5857,7 @@
       <c r="S299" s="4" t="n"/>
       <c r="T299" s="4" t="n"/>
       <c r="U299" s="4" t="n"/>
+      <c r="V299" s="4" t="n"/>
     </row>
     <row r="300">
       <c r="A300" s="4" t="n"/>
@@ -5405,6 +5872,7 @@
       <c r="S300" s="4" t="n"/>
       <c r="T300" s="4" t="n"/>
       <c r="U300" s="4" t="n"/>
+      <c r="V300" s="4" t="n"/>
     </row>
     <row r="301">
       <c r="A301" s="4" t="n"/>
@@ -5419,6 +5887,7 @@
       <c r="S301" s="4" t="n"/>
       <c r="T301" s="4" t="n"/>
       <c r="U301" s="4" t="n"/>
+      <c r="V301" s="4" t="n"/>
     </row>
     <row r="302">
       <c r="A302" s="4" t="n"/>
@@ -5433,6 +5902,7 @@
       <c r="S302" s="4" t="n"/>
       <c r="T302" s="4" t="n"/>
       <c r="U302" s="4" t="n"/>
+      <c r="V302" s="4" t="n"/>
     </row>
     <row r="303">
       <c r="A303" s="4" t="n"/>
@@ -5447,6 +5917,7 @@
       <c r="S303" s="4" t="n"/>
       <c r="T303" s="4" t="n"/>
       <c r="U303" s="4" t="n"/>
+      <c r="V303" s="4" t="n"/>
     </row>
     <row r="304">
       <c r="A304" s="4" t="n"/>
@@ -5461,6 +5932,7 @@
       <c r="S304" s="4" t="n"/>
       <c r="T304" s="4" t="n"/>
       <c r="U304" s="4" t="n"/>
+      <c r="V304" s="4" t="n"/>
     </row>
     <row r="305">
       <c r="A305" s="4" t="n"/>
@@ -5475,6 +5947,7 @@
       <c r="S305" s="4" t="n"/>
       <c r="T305" s="4" t="n"/>
       <c r="U305" s="4" t="n"/>
+      <c r="V305" s="4" t="n"/>
     </row>
     <row r="306">
       <c r="A306" s="4" t="n"/>
@@ -5489,6 +5962,7 @@
       <c r="S306" s="4" t="n"/>
       <c r="T306" s="4" t="n"/>
       <c r="U306" s="4" t="n"/>
+      <c r="V306" s="4" t="n"/>
     </row>
     <row r="307">
       <c r="A307" s="4" t="n"/>
@@ -5503,6 +5977,7 @@
       <c r="S307" s="4" t="n"/>
       <c r="T307" s="4" t="n"/>
       <c r="U307" s="4" t="n"/>
+      <c r="V307" s="4" t="n"/>
     </row>
     <row r="308">
       <c r="A308" s="4" t="n"/>
@@ -5517,6 +5992,7 @@
       <c r="S308" s="4" t="n"/>
       <c r="T308" s="4" t="n"/>
       <c r="U308" s="4" t="n"/>
+      <c r="V308" s="4" t="n"/>
     </row>
     <row r="309">
       <c r="A309" s="4" t="n"/>
@@ -5531,6 +6007,7 @@
       <c r="S309" s="4" t="n"/>
       <c r="T309" s="4" t="n"/>
       <c r="U309" s="4" t="n"/>
+      <c r="V309" s="4" t="n"/>
     </row>
     <row r="310">
       <c r="A310" s="4" t="n"/>
@@ -5545,6 +6022,7 @@
       <c r="S310" s="4" t="n"/>
       <c r="T310" s="4" t="n"/>
       <c r="U310" s="4" t="n"/>
+      <c r="V310" s="4" t="n"/>
     </row>
     <row r="311">
       <c r="A311" s="4" t="n"/>
@@ -5559,6 +6037,7 @@
       <c r="S311" s="4" t="n"/>
       <c r="T311" s="4" t="n"/>
       <c r="U311" s="4" t="n"/>
+      <c r="V311" s="4" t="n"/>
     </row>
     <row r="312">
       <c r="A312" s="4" t="n"/>
@@ -5573,6 +6052,7 @@
       <c r="S312" s="4" t="n"/>
       <c r="T312" s="4" t="n"/>
       <c r="U312" s="4" t="n"/>
+      <c r="V312" s="4" t="n"/>
     </row>
     <row r="313">
       <c r="A313" s="4" t="n"/>
@@ -5587,6 +6067,7 @@
       <c r="S313" s="4" t="n"/>
       <c r="T313" s="4" t="n"/>
       <c r="U313" s="4" t="n"/>
+      <c r="V313" s="4" t="n"/>
     </row>
     <row r="314">
       <c r="A314" s="4" t="n"/>
@@ -5601,6 +6082,7 @@
       <c r="S314" s="4" t="n"/>
       <c r="T314" s="4" t="n"/>
       <c r="U314" s="4" t="n"/>
+      <c r="V314" s="4" t="n"/>
     </row>
     <row r="315">
       <c r="A315" s="4" t="n"/>
@@ -5615,6 +6097,7 @@
       <c r="S315" s="4" t="n"/>
       <c r="T315" s="4" t="n"/>
       <c r="U315" s="4" t="n"/>
+      <c r="V315" s="4" t="n"/>
     </row>
     <row r="316">
       <c r="A316" s="4" t="n"/>
@@ -5629,6 +6112,7 @@
       <c r="S316" s="4" t="n"/>
       <c r="T316" s="4" t="n"/>
       <c r="U316" s="4" t="n"/>
+      <c r="V316" s="4" t="n"/>
     </row>
     <row r="317">
       <c r="A317" s="4" t="n"/>
@@ -5643,6 +6127,7 @@
       <c r="S317" s="4" t="n"/>
       <c r="T317" s="4" t="n"/>
       <c r="U317" s="4" t="n"/>
+      <c r="V317" s="4" t="n"/>
     </row>
     <row r="318">
       <c r="A318" s="4" t="n"/>
@@ -5657,6 +6142,7 @@
       <c r="S318" s="4" t="n"/>
       <c r="T318" s="4" t="n"/>
       <c r="U318" s="4" t="n"/>
+      <c r="V318" s="4" t="n"/>
     </row>
     <row r="319">
       <c r="A319" s="4" t="n"/>
@@ -5671,6 +6157,7 @@
       <c r="S319" s="4" t="n"/>
       <c r="T319" s="4" t="n"/>
       <c r="U319" s="4" t="n"/>
+      <c r="V319" s="4" t="n"/>
     </row>
     <row r="320">
       <c r="A320" s="4" t="n"/>
@@ -5685,6 +6172,7 @@
       <c r="S320" s="4" t="n"/>
       <c r="T320" s="4" t="n"/>
       <c r="U320" s="4" t="n"/>
+      <c r="V320" s="4" t="n"/>
     </row>
     <row r="321">
       <c r="A321" s="4" t="n"/>
@@ -5699,6 +6187,7 @@
       <c r="S321" s="4" t="n"/>
       <c r="T321" s="4" t="n"/>
       <c r="U321" s="4" t="n"/>
+      <c r="V321" s="4" t="n"/>
     </row>
     <row r="322">
       <c r="A322" s="4" t="n"/>
@@ -5713,6 +6202,7 @@
       <c r="S322" s="4" t="n"/>
       <c r="T322" s="4" t="n"/>
       <c r="U322" s="4" t="n"/>
+      <c r="V322" s="4" t="n"/>
     </row>
     <row r="323">
       <c r="A323" s="4" t="n"/>
@@ -5727,6 +6217,7 @@
       <c r="S323" s="4" t="n"/>
       <c r="T323" s="4" t="n"/>
       <c r="U323" s="4" t="n"/>
+      <c r="V323" s="4" t="n"/>
     </row>
     <row r="324">
       <c r="A324" s="4" t="n"/>
@@ -5741,6 +6232,7 @@
       <c r="S324" s="4" t="n"/>
       <c r="T324" s="4" t="n"/>
       <c r="U324" s="4" t="n"/>
+      <c r="V324" s="4" t="n"/>
     </row>
     <row r="325">
       <c r="A325" s="4" t="n"/>
@@ -5755,6 +6247,7 @@
       <c r="S325" s="4" t="n"/>
       <c r="T325" s="4" t="n"/>
       <c r="U325" s="4" t="n"/>
+      <c r="V325" s="4" t="n"/>
     </row>
     <row r="326">
       <c r="A326" s="4" t="n"/>
@@ -5769,6 +6262,7 @@
       <c r="S326" s="4" t="n"/>
       <c r="T326" s="4" t="n"/>
       <c r="U326" s="4" t="n"/>
+      <c r="V326" s="4" t="n"/>
     </row>
     <row r="327">
       <c r="A327" s="4" t="n"/>
@@ -5783,6 +6277,7 @@
       <c r="S327" s="4" t="n"/>
       <c r="T327" s="4" t="n"/>
       <c r="U327" s="4" t="n"/>
+      <c r="V327" s="4" t="n"/>
     </row>
     <row r="328">
       <c r="A328" s="4" t="n"/>
@@ -5797,6 +6292,7 @@
       <c r="S328" s="4" t="n"/>
       <c r="T328" s="4" t="n"/>
       <c r="U328" s="4" t="n"/>
+      <c r="V328" s="4" t="n"/>
     </row>
     <row r="329">
       <c r="A329" s="4" t="n"/>
@@ -5811,6 +6307,7 @@
       <c r="S329" s="4" t="n"/>
       <c r="T329" s="4" t="n"/>
       <c r="U329" s="4" t="n"/>
+      <c r="V329" s="4" t="n"/>
     </row>
     <row r="330">
       <c r="A330" s="4" t="n"/>
@@ -5825,6 +6322,7 @@
       <c r="S330" s="4" t="n"/>
       <c r="T330" s="4" t="n"/>
       <c r="U330" s="4" t="n"/>
+      <c r="V330" s="4" t="n"/>
     </row>
     <row r="331">
       <c r="A331" s="4" t="n"/>
@@ -5839,6 +6337,7 @@
       <c r="S331" s="4" t="n"/>
       <c r="T331" s="4" t="n"/>
       <c r="U331" s="4" t="n"/>
+      <c r="V331" s="4" t="n"/>
     </row>
     <row r="332">
       <c r="A332" s="4" t="n"/>
@@ -5853,6 +6352,7 @@
       <c r="S332" s="4" t="n"/>
       <c r="T332" s="4" t="n"/>
       <c r="U332" s="4" t="n"/>
+      <c r="V332" s="4" t="n"/>
     </row>
     <row r="333">
       <c r="A333" s="4" t="n"/>
@@ -5867,6 +6367,7 @@
       <c r="S333" s="4" t="n"/>
       <c r="T333" s="4" t="n"/>
       <c r="U333" s="4" t="n"/>
+      <c r="V333" s="4" t="n"/>
     </row>
     <row r="334">
       <c r="A334" s="4" t="n"/>
@@ -5881,6 +6382,7 @@
       <c r="S334" s="4" t="n"/>
       <c r="T334" s="4" t="n"/>
       <c r="U334" s="4" t="n"/>
+      <c r="V334" s="4" t="n"/>
     </row>
     <row r="335">
       <c r="A335" s="4" t="n"/>
@@ -5895,6 +6397,7 @@
       <c r="S335" s="4" t="n"/>
       <c r="T335" s="4" t="n"/>
       <c r="U335" s="4" t="n"/>
+      <c r="V335" s="4" t="n"/>
     </row>
     <row r="336">
       <c r="A336" s="4" t="n"/>
@@ -5909,6 +6412,7 @@
       <c r="S336" s="4" t="n"/>
       <c r="T336" s="4" t="n"/>
       <c r="U336" s="4" t="n"/>
+      <c r="V336" s="4" t="n"/>
     </row>
     <row r="337">
       <c r="A337" s="4" t="n"/>
@@ -5923,6 +6427,7 @@
       <c r="S337" s="4" t="n"/>
       <c r="T337" s="4" t="n"/>
       <c r="U337" s="4" t="n"/>
+      <c r="V337" s="4" t="n"/>
     </row>
     <row r="338">
       <c r="A338" s="4" t="n"/>
@@ -5937,6 +6442,7 @@
       <c r="S338" s="4" t="n"/>
       <c r="T338" s="4" t="n"/>
       <c r="U338" s="4" t="n"/>
+      <c r="V338" s="4" t="n"/>
     </row>
     <row r="339">
       <c r="A339" s="4" t="n"/>
@@ -5951,6 +6457,7 @@
       <c r="S339" s="4" t="n"/>
       <c r="T339" s="4" t="n"/>
       <c r="U339" s="4" t="n"/>
+      <c r="V339" s="4" t="n"/>
     </row>
     <row r="340">
       <c r="A340" s="4" t="n"/>
@@ -5965,6 +6472,7 @@
       <c r="S340" s="4" t="n"/>
       <c r="T340" s="4" t="n"/>
       <c r="U340" s="4" t="n"/>
+      <c r="V340" s="4" t="n"/>
     </row>
     <row r="341">
       <c r="A341" s="4" t="n"/>
@@ -5979,6 +6487,7 @@
       <c r="S341" s="4" t="n"/>
       <c r="T341" s="4" t="n"/>
       <c r="U341" s="4" t="n"/>
+      <c r="V341" s="4" t="n"/>
     </row>
     <row r="342">
       <c r="A342" s="4" t="n"/>
@@ -5993,6 +6502,7 @@
       <c r="S342" s="4" t="n"/>
       <c r="T342" s="4" t="n"/>
       <c r="U342" s="4" t="n"/>
+      <c r="V342" s="4" t="n"/>
     </row>
     <row r="343">
       <c r="A343" s="4" t="n"/>
@@ -6007,6 +6517,7 @@
       <c r="S343" s="4" t="n"/>
       <c r="T343" s="4" t="n"/>
       <c r="U343" s="4" t="n"/>
+      <c r="V343" s="4" t="n"/>
     </row>
     <row r="344">
       <c r="A344" s="4" t="n"/>
@@ -6021,6 +6532,7 @@
       <c r="S344" s="4" t="n"/>
       <c r="T344" s="4" t="n"/>
       <c r="U344" s="4" t="n"/>
+      <c r="V344" s="4" t="n"/>
     </row>
     <row r="345">
       <c r="A345" s="4" t="n"/>
@@ -6035,6 +6547,7 @@
       <c r="S345" s="4" t="n"/>
       <c r="T345" s="4" t="n"/>
       <c r="U345" s="4" t="n"/>
+      <c r="V345" s="4" t="n"/>
     </row>
     <row r="346">
       <c r="A346" s="4" t="n"/>
@@ -6049,6 +6562,7 @@
       <c r="S346" s="4" t="n"/>
       <c r="T346" s="4" t="n"/>
       <c r="U346" s="4" t="n"/>
+      <c r="V346" s="4" t="n"/>
     </row>
     <row r="347">
       <c r="A347" s="4" t="n"/>
@@ -6063,6 +6577,7 @@
       <c r="S347" s="4" t="n"/>
       <c r="T347" s="4" t="n"/>
       <c r="U347" s="4" t="n"/>
+      <c r="V347" s="4" t="n"/>
     </row>
     <row r="348">
       <c r="A348" s="4" t="n"/>
@@ -6077,6 +6592,7 @@
       <c r="S348" s="4" t="n"/>
       <c r="T348" s="4" t="n"/>
       <c r="U348" s="4" t="n"/>
+      <c r="V348" s="4" t="n"/>
     </row>
     <row r="349">
       <c r="A349" s="4" t="n"/>
@@ -6091,6 +6607,7 @@
       <c r="S349" s="4" t="n"/>
       <c r="T349" s="4" t="n"/>
       <c r="U349" s="4" t="n"/>
+      <c r="V349" s="4" t="n"/>
     </row>
     <row r="350">
       <c r="A350" s="4" t="n"/>
@@ -6105,6 +6622,7 @@
       <c r="S350" s="4" t="n"/>
       <c r="T350" s="4" t="n"/>
       <c r="U350" s="4" t="n"/>
+      <c r="V350" s="4" t="n"/>
     </row>
     <row r="351">
       <c r="A351" s="4" t="n"/>
@@ -6119,6 +6637,7 @@
       <c r="S351" s="4" t="n"/>
       <c r="T351" s="4" t="n"/>
       <c r="U351" s="4" t="n"/>
+      <c r="V351" s="4" t="n"/>
     </row>
     <row r="352">
       <c r="A352" s="4" t="n"/>
@@ -6133,6 +6652,7 @@
       <c r="S352" s="4" t="n"/>
       <c r="T352" s="4" t="n"/>
       <c r="U352" s="4" t="n"/>
+      <c r="V352" s="4" t="n"/>
     </row>
     <row r="353">
       <c r="A353" s="4" t="n"/>
@@ -6147,6 +6667,7 @@
       <c r="S353" s="4" t="n"/>
       <c r="T353" s="4" t="n"/>
       <c r="U353" s="4" t="n"/>
+      <c r="V353" s="4" t="n"/>
     </row>
     <row r="354">
       <c r="A354" s="4" t="n"/>
@@ -6161,6 +6682,7 @@
       <c r="S354" s="4" t="n"/>
       <c r="T354" s="4" t="n"/>
       <c r="U354" s="4" t="n"/>
+      <c r="V354" s="4" t="n"/>
     </row>
     <row r="355">
       <c r="A355" s="4" t="n"/>
@@ -6175,6 +6697,7 @@
       <c r="S355" s="4" t="n"/>
       <c r="T355" s="4" t="n"/>
       <c r="U355" s="4" t="n"/>
+      <c r="V355" s="4" t="n"/>
     </row>
     <row r="356">
       <c r="A356" s="4" t="n"/>
@@ -6189,6 +6712,7 @@
       <c r="S356" s="4" t="n"/>
       <c r="T356" s="4" t="n"/>
       <c r="U356" s="4" t="n"/>
+      <c r="V356" s="4" t="n"/>
     </row>
     <row r="357">
       <c r="A357" s="4" t="n"/>
@@ -6203,6 +6727,7 @@
       <c r="S357" s="4" t="n"/>
       <c r="T357" s="4" t="n"/>
       <c r="U357" s="4" t="n"/>
+      <c r="V357" s="4" t="n"/>
     </row>
     <row r="358">
       <c r="A358" s="4" t="n"/>
@@ -6217,6 +6742,7 @@
       <c r="S358" s="4" t="n"/>
       <c r="T358" s="4" t="n"/>
       <c r="U358" s="4" t="n"/>
+      <c r="V358" s="4" t="n"/>
     </row>
     <row r="359">
       <c r="A359" s="4" t="n"/>
@@ -6231,6 +6757,7 @@
       <c r="S359" s="4" t="n"/>
       <c r="T359" s="4" t="n"/>
       <c r="U359" s="4" t="n"/>
+      <c r="V359" s="4" t="n"/>
     </row>
     <row r="360">
       <c r="A360" s="4" t="n"/>
@@ -6245,6 +6772,7 @@
       <c r="S360" s="4" t="n"/>
       <c r="T360" s="4" t="n"/>
       <c r="U360" s="4" t="n"/>
+      <c r="V360" s="4" t="n"/>
     </row>
     <row r="361">
       <c r="A361" s="4" t="n"/>
@@ -6259,6 +6787,7 @@
       <c r="S361" s="4" t="n"/>
       <c r="T361" s="4" t="n"/>
       <c r="U361" s="4" t="n"/>
+      <c r="V361" s="4" t="n"/>
     </row>
     <row r="362">
       <c r="A362" s="4" t="n"/>
@@ -6273,6 +6802,7 @@
       <c r="S362" s="4" t="n"/>
       <c r="T362" s="4" t="n"/>
       <c r="U362" s="4" t="n"/>
+      <c r="V362" s="4" t="n"/>
     </row>
     <row r="363">
       <c r="A363" s="4" t="n"/>
@@ -6287,6 +6817,7 @@
       <c r="S363" s="4" t="n"/>
       <c r="T363" s="4" t="n"/>
       <c r="U363" s="4" t="n"/>
+      <c r="V363" s="4" t="n"/>
     </row>
     <row r="364">
       <c r="A364" s="4" t="n"/>
@@ -6301,6 +6832,7 @@
       <c r="S364" s="4" t="n"/>
       <c r="T364" s="4" t="n"/>
       <c r="U364" s="4" t="n"/>
+      <c r="V364" s="4" t="n"/>
     </row>
     <row r="365">
       <c r="A365" s="4" t="n"/>
@@ -6315,6 +6847,7 @@
       <c r="S365" s="4" t="n"/>
       <c r="T365" s="4" t="n"/>
       <c r="U365" s="4" t="n"/>
+      <c r="V365" s="4" t="n"/>
     </row>
     <row r="366">
       <c r="A366" s="4" t="n"/>
@@ -6329,6 +6862,7 @@
       <c r="S366" s="4" t="n"/>
       <c r="T366" s="4" t="n"/>
       <c r="U366" s="4" t="n"/>
+      <c r="V366" s="4" t="n"/>
     </row>
     <row r="367">
       <c r="A367" s="4" t="n"/>
@@ -6343,6 +6877,7 @@
       <c r="S367" s="4" t="n"/>
       <c r="T367" s="4" t="n"/>
       <c r="U367" s="4" t="n"/>
+      <c r="V367" s="4" t="n"/>
     </row>
     <row r="368">
       <c r="A368" s="4" t="n"/>
@@ -6357,6 +6892,7 @@
       <c r="S368" s="4" t="n"/>
       <c r="T368" s="4" t="n"/>
       <c r="U368" s="4" t="n"/>
+      <c r="V368" s="4" t="n"/>
     </row>
     <row r="369">
       <c r="A369" s="4" t="n"/>
@@ -6371,6 +6907,7 @@
       <c r="S369" s="4" t="n"/>
       <c r="T369" s="4" t="n"/>
       <c r="U369" s="4" t="n"/>
+      <c r="V369" s="4" t="n"/>
     </row>
     <row r="370">
       <c r="A370" s="4" t="n"/>
@@ -6385,6 +6922,7 @@
       <c r="S370" s="4" t="n"/>
       <c r="T370" s="4" t="n"/>
       <c r="U370" s="4" t="n"/>
+      <c r="V370" s="4" t="n"/>
     </row>
     <row r="371">
       <c r="A371" s="4" t="n"/>
@@ -6399,6 +6937,7 @@
       <c r="S371" s="4" t="n"/>
       <c r="T371" s="4" t="n"/>
       <c r="U371" s="4" t="n"/>
+      <c r="V371" s="4" t="n"/>
     </row>
     <row r="372">
       <c r="A372" s="4" t="n"/>
@@ -6413,6 +6952,7 @@
       <c r="S372" s="4" t="n"/>
       <c r="T372" s="4" t="n"/>
       <c r="U372" s="4" t="n"/>
+      <c r="V372" s="4" t="n"/>
     </row>
     <row r="373">
       <c r="A373" s="4" t="n"/>
@@ -6427,6 +6967,7 @@
       <c r="S373" s="4" t="n"/>
       <c r="T373" s="4" t="n"/>
       <c r="U373" s="4" t="n"/>
+      <c r="V373" s="4" t="n"/>
     </row>
     <row r="374">
       <c r="A374" s="4" t="n"/>
@@ -6441,6 +6982,7 @@
       <c r="S374" s="4" t="n"/>
       <c r="T374" s="4" t="n"/>
       <c r="U374" s="4" t="n"/>
+      <c r="V374" s="4" t="n"/>
     </row>
     <row r="375">
       <c r="A375" s="4" t="n"/>
@@ -6455,6 +6997,7 @@
       <c r="S375" s="4" t="n"/>
       <c r="T375" s="4" t="n"/>
       <c r="U375" s="4" t="n"/>
+      <c r="V375" s="4" t="n"/>
     </row>
     <row r="376">
       <c r="A376" s="4" t="n"/>
@@ -6469,6 +7012,7 @@
       <c r="S376" s="4" t="n"/>
       <c r="T376" s="4" t="n"/>
       <c r="U376" s="4" t="n"/>
+      <c r="V376" s="4" t="n"/>
     </row>
     <row r="377">
       <c r="A377" s="4" t="n"/>
@@ -6483,6 +7027,7 @@
       <c r="S377" s="4" t="n"/>
       <c r="T377" s="4" t="n"/>
       <c r="U377" s="4" t="n"/>
+      <c r="V377" s="4" t="n"/>
     </row>
     <row r="378">
       <c r="A378" s="4" t="n"/>
@@ -6497,6 +7042,7 @@
       <c r="S378" s="4" t="n"/>
       <c r="T378" s="4" t="n"/>
       <c r="U378" s="4" t="n"/>
+      <c r="V378" s="4" t="n"/>
     </row>
     <row r="379">
       <c r="A379" s="4" t="n"/>
@@ -6511,6 +7057,7 @@
       <c r="S379" s="4" t="n"/>
       <c r="T379" s="4" t="n"/>
       <c r="U379" s="4" t="n"/>
+      <c r="V379" s="4" t="n"/>
     </row>
     <row r="380">
       <c r="A380" s="4" t="n"/>
@@ -6525,6 +7072,7 @@
       <c r="S380" s="4" t="n"/>
       <c r="T380" s="4" t="n"/>
       <c r="U380" s="4" t="n"/>
+      <c r="V380" s="4" t="n"/>
     </row>
     <row r="381">
       <c r="A381" s="4" t="n"/>
@@ -6539,6 +7087,7 @@
       <c r="S381" s="4" t="n"/>
       <c r="T381" s="4" t="n"/>
       <c r="U381" s="4" t="n"/>
+      <c r="V381" s="4" t="n"/>
     </row>
     <row r="382">
       <c r="A382" s="4" t="n"/>
@@ -6553,6 +7102,7 @@
       <c r="S382" s="4" t="n"/>
       <c r="T382" s="4" t="n"/>
       <c r="U382" s="4" t="n"/>
+      <c r="V382" s="4" t="n"/>
     </row>
     <row r="383">
       <c r="A383" s="4" t="n"/>
@@ -6567,6 +7117,7 @@
       <c r="S383" s="4" t="n"/>
       <c r="T383" s="4" t="n"/>
       <c r="U383" s="4" t="n"/>
+      <c r="V383" s="4" t="n"/>
     </row>
     <row r="384">
       <c r="A384" s="4" t="n"/>
@@ -6581,6 +7132,7 @@
       <c r="S384" s="4" t="n"/>
       <c r="T384" s="4" t="n"/>
       <c r="U384" s="4" t="n"/>
+      <c r="V384" s="4" t="n"/>
     </row>
     <row r="385">
       <c r="A385" s="4" t="n"/>
@@ -6595,6 +7147,7 @@
       <c r="S385" s="4" t="n"/>
       <c r="T385" s="4" t="n"/>
       <c r="U385" s="4" t="n"/>
+      <c r="V385" s="4" t="n"/>
     </row>
     <row r="386">
       <c r="A386" s="4" t="n"/>
@@ -6609,6 +7162,7 @@
       <c r="S386" s="4" t="n"/>
       <c r="T386" s="4" t="n"/>
       <c r="U386" s="4" t="n"/>
+      <c r="V386" s="4" t="n"/>
     </row>
     <row r="387">
       <c r="A387" s="4" t="n"/>
@@ -6623,6 +7177,7 @@
       <c r="S387" s="4" t="n"/>
       <c r="T387" s="4" t="n"/>
       <c r="U387" s="4" t="n"/>
+      <c r="V387" s="4" t="n"/>
     </row>
     <row r="388">
       <c r="A388" s="4" t="n"/>
@@ -6637,6 +7192,7 @@
       <c r="S388" s="4" t="n"/>
       <c r="T388" s="4" t="n"/>
       <c r="U388" s="4" t="n"/>
+      <c r="V388" s="4" t="n"/>
     </row>
     <row r="389">
       <c r="A389" s="4" t="n"/>
@@ -6651,6 +7207,7 @@
       <c r="S389" s="4" t="n"/>
       <c r="T389" s="4" t="n"/>
       <c r="U389" s="4" t="n"/>
+      <c r="V389" s="4" t="n"/>
     </row>
     <row r="390">
       <c r="A390" s="4" t="n"/>
@@ -6665,6 +7222,7 @@
       <c r="S390" s="4" t="n"/>
       <c r="T390" s="4" t="n"/>
       <c r="U390" s="4" t="n"/>
+      <c r="V390" s="4" t="n"/>
     </row>
     <row r="391">
       <c r="A391" s="4" t="n"/>
@@ -6679,6 +7237,7 @@
       <c r="S391" s="4" t="n"/>
       <c r="T391" s="4" t="n"/>
       <c r="U391" s="4" t="n"/>
+      <c r="V391" s="4" t="n"/>
     </row>
     <row r="392">
       <c r="A392" s="4" t="n"/>
@@ -6693,6 +7252,7 @@
       <c r="S392" s="4" t="n"/>
       <c r="T392" s="4" t="n"/>
       <c r="U392" s="4" t="n"/>
+      <c r="V392" s="4" t="n"/>
     </row>
     <row r="393">
       <c r="A393" s="4" t="n"/>
@@ -6707,6 +7267,7 @@
       <c r="S393" s="4" t="n"/>
       <c r="T393" s="4" t="n"/>
       <c r="U393" s="4" t="n"/>
+      <c r="V393" s="4" t="n"/>
     </row>
     <row r="394">
       <c r="A394" s="4" t="n"/>
@@ -6721,6 +7282,7 @@
       <c r="S394" s="4" t="n"/>
       <c r="T394" s="4" t="n"/>
       <c r="U394" s="4" t="n"/>
+      <c r="V394" s="4" t="n"/>
     </row>
     <row r="395">
       <c r="A395" s="4" t="n"/>
@@ -6735,6 +7297,7 @@
       <c r="S395" s="4" t="n"/>
       <c r="T395" s="4" t="n"/>
       <c r="U395" s="4" t="n"/>
+      <c r="V395" s="4" t="n"/>
     </row>
     <row r="396">
       <c r="A396" s="4" t="n"/>
@@ -6749,6 +7312,7 @@
       <c r="S396" s="4" t="n"/>
       <c r="T396" s="4" t="n"/>
       <c r="U396" s="4" t="n"/>
+      <c r="V396" s="4" t="n"/>
     </row>
     <row r="397">
       <c r="A397" s="4" t="n"/>
@@ -6763,6 +7327,7 @@
       <c r="S397" s="4" t="n"/>
       <c r="T397" s="4" t="n"/>
       <c r="U397" s="4" t="n"/>
+      <c r="V397" s="4" t="n"/>
     </row>
     <row r="398">
       <c r="A398" s="4" t="n"/>
@@ -6777,6 +7342,7 @@
       <c r="S398" s="4" t="n"/>
       <c r="T398" s="4" t="n"/>
       <c r="U398" s="4" t="n"/>
+      <c r="V398" s="4" t="n"/>
     </row>
     <row r="399">
       <c r="A399" s="4" t="n"/>
@@ -6791,6 +7357,7 @@
       <c r="S399" s="4" t="n"/>
       <c r="T399" s="4" t="n"/>
       <c r="U399" s="4" t="n"/>
+      <c r="V399" s="4" t="n"/>
     </row>
     <row r="400">
       <c r="A400" s="4" t="n"/>
@@ -6805,6 +7372,7 @@
       <c r="S400" s="4" t="n"/>
       <c r="T400" s="4" t="n"/>
       <c r="U400" s="4" t="n"/>
+      <c r="V400" s="4" t="n"/>
     </row>
     <row r="401">
       <c r="A401" s="4" t="n"/>
@@ -6819,6 +7387,7 @@
       <c r="S401" s="4" t="n"/>
       <c r="T401" s="4" t="n"/>
       <c r="U401" s="4" t="n"/>
+      <c r="V401" s="4" t="n"/>
     </row>
     <row r="402">
       <c r="A402" s="4" t="n"/>
@@ -6833,6 +7402,7 @@
       <c r="S402" s="4" t="n"/>
       <c r="T402" s="4" t="n"/>
       <c r="U402" s="4" t="n"/>
+      <c r="V402" s="4" t="n"/>
     </row>
     <row r="403">
       <c r="A403" s="4" t="n"/>
@@ -6847,6 +7417,7 @@
       <c r="S403" s="4" t="n"/>
       <c r="T403" s="4" t="n"/>
       <c r="U403" s="4" t="n"/>
+      <c r="V403" s="4" t="n"/>
     </row>
     <row r="404">
       <c r="A404" s="4" t="n"/>
@@ -6861,6 +7432,7 @@
       <c r="S404" s="4" t="n"/>
       <c r="T404" s="4" t="n"/>
       <c r="U404" s="4" t="n"/>
+      <c r="V404" s="4" t="n"/>
     </row>
     <row r="405">
       <c r="A405" s="4" t="n"/>
@@ -6875,6 +7447,7 @@
       <c r="S405" s="4" t="n"/>
       <c r="T405" s="4" t="n"/>
       <c r="U405" s="4" t="n"/>
+      <c r="V405" s="4" t="n"/>
     </row>
     <row r="406">
       <c r="A406" s="4" t="n"/>
@@ -6889,6 +7462,7 @@
       <c r="S406" s="4" t="n"/>
       <c r="T406" s="4" t="n"/>
       <c r="U406" s="4" t="n"/>
+      <c r="V406" s="4" t="n"/>
     </row>
     <row r="407">
       <c r="A407" s="4" t="n"/>
@@ -6903,6 +7477,7 @@
       <c r="S407" s="4" t="n"/>
       <c r="T407" s="4" t="n"/>
       <c r="U407" s="4" t="n"/>
+      <c r="V407" s="4" t="n"/>
     </row>
     <row r="408">
       <c r="A408" s="4" t="n"/>
@@ -6917,6 +7492,7 @@
       <c r="S408" s="4" t="n"/>
       <c r="T408" s="4" t="n"/>
       <c r="U408" s="4" t="n"/>
+      <c r="V408" s="4" t="n"/>
     </row>
     <row r="409">
       <c r="A409" s="4" t="n"/>
@@ -6931,6 +7507,7 @@
       <c r="S409" s="4" t="n"/>
       <c r="T409" s="4" t="n"/>
       <c r="U409" s="4" t="n"/>
+      <c r="V409" s="4" t="n"/>
     </row>
     <row r="410">
       <c r="A410" s="4" t="n"/>
@@ -6945,6 +7522,7 @@
       <c r="S410" s="4" t="n"/>
       <c r="T410" s="4" t="n"/>
       <c r="U410" s="4" t="n"/>
+      <c r="V410" s="4" t="n"/>
     </row>
     <row r="411">
       <c r="A411" s="4" t="n"/>
@@ -6959,6 +7537,7 @@
       <c r="S411" s="4" t="n"/>
       <c r="T411" s="4" t="n"/>
       <c r="U411" s="4" t="n"/>
+      <c r="V411" s="4" t="n"/>
     </row>
     <row r="412">
       <c r="A412" s="4" t="n"/>
@@ -6973,6 +7552,7 @@
       <c r="S412" s="4" t="n"/>
       <c r="T412" s="4" t="n"/>
       <c r="U412" s="4" t="n"/>
+      <c r="V412" s="4" t="n"/>
     </row>
     <row r="413">
       <c r="A413" s="4" t="n"/>
@@ -6987,6 +7567,7 @@
       <c r="S413" s="4" t="n"/>
       <c r="T413" s="4" t="n"/>
       <c r="U413" s="4" t="n"/>
+      <c r="V413" s="4" t="n"/>
     </row>
     <row r="414">
       <c r="A414" s="4" t="n"/>
@@ -7001,6 +7582,7 @@
       <c r="S414" s="4" t="n"/>
       <c r="T414" s="4" t="n"/>
       <c r="U414" s="4" t="n"/>
+      <c r="V414" s="4" t="n"/>
     </row>
     <row r="415">
       <c r="A415" s="4" t="n"/>
@@ -7015,6 +7597,7 @@
       <c r="S415" s="4" t="n"/>
       <c r="T415" s="4" t="n"/>
       <c r="U415" s="4" t="n"/>
+      <c r="V415" s="4" t="n"/>
     </row>
     <row r="416">
       <c r="A416" s="4" t="n"/>
@@ -7029,6 +7612,7 @@
       <c r="S416" s="4" t="n"/>
       <c r="T416" s="4" t="n"/>
       <c r="U416" s="4" t="n"/>
+      <c r="V416" s="4" t="n"/>
     </row>
     <row r="417">
       <c r="A417" s="4" t="n"/>
@@ -7043,6 +7627,7 @@
       <c r="S417" s="4" t="n"/>
       <c r="T417" s="4" t="n"/>
       <c r="U417" s="4" t="n"/>
+      <c r="V417" s="4" t="n"/>
     </row>
     <row r="418">
       <c r="A418" s="4" t="n"/>
@@ -7057,6 +7642,7 @@
       <c r="S418" s="4" t="n"/>
       <c r="T418" s="4" t="n"/>
       <c r="U418" s="4" t="n"/>
+      <c r="V418" s="4" t="n"/>
     </row>
     <row r="419">
       <c r="A419" s="4" t="n"/>
@@ -7071,6 +7657,7 @@
       <c r="S419" s="4" t="n"/>
       <c r="T419" s="4" t="n"/>
       <c r="U419" s="4" t="n"/>
+      <c r="V419" s="4" t="n"/>
     </row>
     <row r="420">
       <c r="A420" s="4" t="n"/>
@@ -7085,6 +7672,7 @@
       <c r="S420" s="4" t="n"/>
       <c r="T420" s="4" t="n"/>
       <c r="U420" s="4" t="n"/>
+      <c r="V420" s="4" t="n"/>
     </row>
     <row r="421">
       <c r="A421" s="4" t="n"/>
@@ -7099,6 +7687,7 @@
       <c r="S421" s="4" t="n"/>
       <c r="T421" s="4" t="n"/>
       <c r="U421" s="4" t="n"/>
+      <c r="V421" s="4" t="n"/>
     </row>
     <row r="422">
       <c r="A422" s="4" t="n"/>
@@ -7113,6 +7702,7 @@
       <c r="S422" s="4" t="n"/>
       <c r="T422" s="4" t="n"/>
       <c r="U422" s="4" t="n"/>
+      <c r="V422" s="4" t="n"/>
     </row>
     <row r="423">
       <c r="A423" s="4" t="n"/>
@@ -7127,6 +7717,7 @@
       <c r="S423" s="4" t="n"/>
       <c r="T423" s="4" t="n"/>
       <c r="U423" s="4" t="n"/>
+      <c r="V423" s="4" t="n"/>
     </row>
     <row r="424">
       <c r="A424" s="4" t="n"/>
@@ -7141,6 +7732,7 @@
       <c r="S424" s="4" t="n"/>
       <c r="T424" s="4" t="n"/>
       <c r="U424" s="4" t="n"/>
+      <c r="V424" s="4" t="n"/>
     </row>
     <row r="425">
       <c r="A425" s="4" t="n"/>
@@ -7155,6 +7747,7 @@
       <c r="S425" s="4" t="n"/>
       <c r="T425" s="4" t="n"/>
       <c r="U425" s="4" t="n"/>
+      <c r="V425" s="4" t="n"/>
     </row>
     <row r="426">
       <c r="A426" s="4" t="n"/>
@@ -7169,6 +7762,7 @@
       <c r="S426" s="4" t="n"/>
       <c r="T426" s="4" t="n"/>
       <c r="U426" s="4" t="n"/>
+      <c r="V426" s="4" t="n"/>
     </row>
     <row r="427">
       <c r="A427" s="4" t="n"/>
@@ -7183,6 +7777,7 @@
       <c r="S427" s="4" t="n"/>
       <c r="T427" s="4" t="n"/>
       <c r="U427" s="4" t="n"/>
+      <c r="V427" s="4" t="n"/>
     </row>
     <row r="428">
       <c r="A428" s="4" t="n"/>
@@ -7197,6 +7792,7 @@
       <c r="S428" s="4" t="n"/>
       <c r="T428" s="4" t="n"/>
       <c r="U428" s="4" t="n"/>
+      <c r="V428" s="4" t="n"/>
     </row>
     <row r="429">
       <c r="A429" s="4" t="n"/>
@@ -7211,6 +7807,7 @@
       <c r="S429" s="4" t="n"/>
       <c r="T429" s="4" t="n"/>
       <c r="U429" s="4" t="n"/>
+      <c r="V429" s="4" t="n"/>
     </row>
     <row r="430">
       <c r="A430" s="4" t="n"/>
@@ -7225,6 +7822,7 @@
       <c r="S430" s="4" t="n"/>
       <c r="T430" s="4" t="n"/>
       <c r="U430" s="4" t="n"/>
+      <c r="V430" s="4" t="n"/>
     </row>
     <row r="431">
       <c r="A431" s="4" t="n"/>
@@ -7239,6 +7837,7 @@
       <c r="S431" s="4" t="n"/>
       <c r="T431" s="4" t="n"/>
       <c r="U431" s="4" t="n"/>
+      <c r="V431" s="4" t="n"/>
     </row>
     <row r="432">
       <c r="A432" s="4" t="n"/>
@@ -7253,6 +7852,7 @@
       <c r="S432" s="4" t="n"/>
       <c r="T432" s="4" t="n"/>
       <c r="U432" s="4" t="n"/>
+      <c r="V432" s="4" t="n"/>
     </row>
     <row r="433">
       <c r="A433" s="4" t="n"/>
@@ -7267,6 +7867,7 @@
       <c r="S433" s="4" t="n"/>
       <c r="T433" s="4" t="n"/>
       <c r="U433" s="4" t="n"/>
+      <c r="V433" s="4" t="n"/>
     </row>
     <row r="434">
       <c r="A434" s="4" t="n"/>
@@ -7281,6 +7882,7 @@
       <c r="S434" s="4" t="n"/>
       <c r="T434" s="4" t="n"/>
       <c r="U434" s="4" t="n"/>
+      <c r="V434" s="4" t="n"/>
     </row>
     <row r="435">
       <c r="A435" s="4" t="n"/>
@@ -7295,6 +7897,7 @@
       <c r="S435" s="4" t="n"/>
       <c r="T435" s="4" t="n"/>
       <c r="U435" s="4" t="n"/>
+      <c r="V435" s="4" t="n"/>
     </row>
     <row r="436">
       <c r="A436" s="4" t="n"/>
@@ -7309,6 +7912,7 @@
       <c r="S436" s="4" t="n"/>
       <c r="T436" s="4" t="n"/>
       <c r="U436" s="4" t="n"/>
+      <c r="V436" s="4" t="n"/>
     </row>
     <row r="437">
       <c r="A437" s="4" t="n"/>
@@ -7323,6 +7927,7 @@
       <c r="S437" s="4" t="n"/>
       <c r="T437" s="4" t="n"/>
       <c r="U437" s="4" t="n"/>
+      <c r="V437" s="4" t="n"/>
     </row>
     <row r="438">
       <c r="A438" s="4" t="n"/>
@@ -7337,6 +7942,7 @@
       <c r="S438" s="4" t="n"/>
       <c r="T438" s="4" t="n"/>
       <c r="U438" s="4" t="n"/>
+      <c r="V438" s="4" t="n"/>
     </row>
     <row r="439">
       <c r="A439" s="4" t="n"/>
@@ -7351,6 +7957,7 @@
       <c r="S439" s="4" t="n"/>
       <c r="T439" s="4" t="n"/>
       <c r="U439" s="4" t="n"/>
+      <c r="V439" s="4" t="n"/>
     </row>
     <row r="440">
       <c r="A440" s="4" t="n"/>
@@ -7365,6 +7972,7 @@
       <c r="S440" s="4" t="n"/>
       <c r="T440" s="4" t="n"/>
       <c r="U440" s="4" t="n"/>
+      <c r="V440" s="4" t="n"/>
     </row>
     <row r="441">
       <c r="A441" s="4" t="n"/>
@@ -7379,6 +7987,7 @@
       <c r="S441" s="4" t="n"/>
       <c r="T441" s="4" t="n"/>
       <c r="U441" s="4" t="n"/>
+      <c r="V441" s="4" t="n"/>
     </row>
     <row r="442">
       <c r="A442" s="4" t="n"/>
@@ -7393,6 +8002,7 @@
       <c r="S442" s="4" t="n"/>
       <c r="T442" s="4" t="n"/>
       <c r="U442" s="4" t="n"/>
+      <c r="V442" s="4" t="n"/>
     </row>
     <row r="443">
       <c r="A443" s="4" t="n"/>
@@ -7407,6 +8017,7 @@
       <c r="S443" s="4" t="n"/>
       <c r="T443" s="4" t="n"/>
       <c r="U443" s="4" t="n"/>
+      <c r="V443" s="4" t="n"/>
     </row>
     <row r="444">
       <c r="A444" s="4" t="n"/>
@@ -7421,6 +8032,7 @@
       <c r="S444" s="4" t="n"/>
       <c r="T444" s="4" t="n"/>
       <c r="U444" s="4" t="n"/>
+      <c r="V444" s="4" t="n"/>
     </row>
     <row r="445">
       <c r="A445" s="4" t="n"/>
@@ -7435,6 +8047,7 @@
       <c r="S445" s="4" t="n"/>
       <c r="T445" s="4" t="n"/>
       <c r="U445" s="4" t="n"/>
+      <c r="V445" s="4" t="n"/>
     </row>
     <row r="446">
       <c r="A446" s="4" t="n"/>
@@ -7449,6 +8062,7 @@
       <c r="S446" s="4" t="n"/>
       <c r="T446" s="4" t="n"/>
       <c r="U446" s="4" t="n"/>
+      <c r="V446" s="4" t="n"/>
     </row>
     <row r="447">
       <c r="A447" s="4" t="n"/>
@@ -7463,6 +8077,7 @@
       <c r="S447" s="4" t="n"/>
       <c r="T447" s="4" t="n"/>
       <c r="U447" s="4" t="n"/>
+      <c r="V447" s="4" t="n"/>
     </row>
     <row r="448">
       <c r="A448" s="4" t="n"/>
@@ -7477,6 +8092,7 @@
       <c r="S448" s="4" t="n"/>
       <c r="T448" s="4" t="n"/>
       <c r="U448" s="4" t="n"/>
+      <c r="V448" s="4" t="n"/>
     </row>
     <row r="449">
       <c r="A449" s="4" t="n"/>
@@ -7491,6 +8107,7 @@
       <c r="S449" s="4" t="n"/>
       <c r="T449" s="4" t="n"/>
       <c r="U449" s="4" t="n"/>
+      <c r="V449" s="4" t="n"/>
     </row>
     <row r="450">
       <c r="A450" s="4" t="n"/>
@@ -7505,6 +8122,7 @@
       <c r="S450" s="4" t="n"/>
       <c r="T450" s="4" t="n"/>
       <c r="U450" s="4" t="n"/>
+      <c r="V450" s="4" t="n"/>
     </row>
     <row r="451">
       <c r="A451" s="4" t="n"/>
@@ -7519,6 +8137,7 @@
       <c r="S451" s="4" t="n"/>
       <c r="T451" s="4" t="n"/>
       <c r="U451" s="4" t="n"/>
+      <c r="V451" s="4" t="n"/>
     </row>
     <row r="452">
       <c r="A452" s="4" t="n"/>
@@ -7533,6 +8152,7 @@
       <c r="S452" s="4" t="n"/>
       <c r="T452" s="4" t="n"/>
       <c r="U452" s="4" t="n"/>
+      <c r="V452" s="4" t="n"/>
     </row>
     <row r="453">
       <c r="A453" s="4" t="n"/>
@@ -7547,6 +8167,7 @@
       <c r="S453" s="4" t="n"/>
       <c r="T453" s="4" t="n"/>
       <c r="U453" s="4" t="n"/>
+      <c r="V453" s="4" t="n"/>
     </row>
     <row r="454">
       <c r="A454" s="4" t="n"/>
@@ -7561,6 +8182,7 @@
       <c r="S454" s="4" t="n"/>
       <c r="T454" s="4" t="n"/>
       <c r="U454" s="4" t="n"/>
+      <c r="V454" s="4" t="n"/>
     </row>
     <row r="455">
       <c r="A455" s="4" t="n"/>
@@ -7575,6 +8197,7 @@
       <c r="S455" s="4" t="n"/>
       <c r="T455" s="4" t="n"/>
       <c r="U455" s="4" t="n"/>
+      <c r="V455" s="4" t="n"/>
     </row>
     <row r="456">
       <c r="A456" s="4" t="n"/>
@@ -7589,6 +8212,7 @@
       <c r="S456" s="4" t="n"/>
       <c r="T456" s="4" t="n"/>
       <c r="U456" s="4" t="n"/>
+      <c r="V456" s="4" t="n"/>
     </row>
     <row r="457">
       <c r="A457" s="4" t="n"/>
@@ -7603,6 +8227,7 @@
       <c r="S457" s="4" t="n"/>
       <c r="T457" s="4" t="n"/>
       <c r="U457" s="4" t="n"/>
+      <c r="V457" s="4" t="n"/>
     </row>
     <row r="458">
       <c r="A458" s="4" t="n"/>
@@ -7617,6 +8242,7 @@
       <c r="S458" s="4" t="n"/>
       <c r="T458" s="4" t="n"/>
       <c r="U458" s="4" t="n"/>
+      <c r="V458" s="4" t="n"/>
     </row>
     <row r="459">
       <c r="A459" s="4" t="n"/>
@@ -7631,6 +8257,7 @@
       <c r="S459" s="4" t="n"/>
       <c r="T459" s="4" t="n"/>
       <c r="U459" s="4" t="n"/>
+      <c r="V459" s="4" t="n"/>
     </row>
     <row r="460">
       <c r="A460" s="4" t="n"/>
@@ -7645,6 +8272,7 @@
       <c r="S460" s="4" t="n"/>
       <c r="T460" s="4" t="n"/>
       <c r="U460" s="4" t="n"/>
+      <c r="V460" s="4" t="n"/>
     </row>
     <row r="461">
       <c r="A461" s="4" t="n"/>
@@ -7659,6 +8287,7 @@
       <c r="S461" s="4" t="n"/>
       <c r="T461" s="4" t="n"/>
       <c r="U461" s="4" t="n"/>
+      <c r="V461" s="4" t="n"/>
     </row>
     <row r="462">
       <c r="A462" s="4" t="n"/>
@@ -7673,6 +8302,7 @@
       <c r="S462" s="4" t="n"/>
       <c r="T462" s="4" t="n"/>
       <c r="U462" s="4" t="n"/>
+      <c r="V462" s="4" t="n"/>
     </row>
     <row r="463">
       <c r="A463" s="4" t="n"/>
@@ -7687,6 +8317,7 @@
       <c r="S463" s="4" t="n"/>
       <c r="T463" s="4" t="n"/>
       <c r="U463" s="4" t="n"/>
+      <c r="V463" s="4" t="n"/>
     </row>
     <row r="464">
       <c r="A464" s="4" t="n"/>
@@ -7701,6 +8332,7 @@
       <c r="S464" s="4" t="n"/>
       <c r="T464" s="4" t="n"/>
       <c r="U464" s="4" t="n"/>
+      <c r="V464" s="4" t="n"/>
     </row>
     <row r="465">
       <c r="A465" s="4" t="n"/>
@@ -7715,6 +8347,7 @@
       <c r="S465" s="4" t="n"/>
       <c r="T465" s="4" t="n"/>
       <c r="U465" s="4" t="n"/>
+      <c r="V465" s="4" t="n"/>
     </row>
     <row r="466">
       <c r="A466" s="4" t="n"/>
@@ -7729,6 +8362,7 @@
       <c r="S466" s="4" t="n"/>
       <c r="T466" s="4" t="n"/>
       <c r="U466" s="4" t="n"/>
+      <c r="V466" s="4" t="n"/>
     </row>
     <row r="467">
       <c r="A467" s="4" t="n"/>
@@ -7743,6 +8377,7 @@
       <c r="S467" s="4" t="n"/>
       <c r="T467" s="4" t="n"/>
       <c r="U467" s="4" t="n"/>
+      <c r="V467" s="4" t="n"/>
     </row>
     <row r="468">
       <c r="A468" s="4" t="n"/>
@@ -7757,6 +8392,7 @@
       <c r="S468" s="4" t="n"/>
       <c r="T468" s="4" t="n"/>
       <c r="U468" s="4" t="n"/>
+      <c r="V468" s="4" t="n"/>
     </row>
     <row r="469">
       <c r="A469" s="4" t="n"/>
@@ -7771,6 +8407,7 @@
       <c r="S469" s="4" t="n"/>
       <c r="T469" s="4" t="n"/>
       <c r="U469" s="4" t="n"/>
+      <c r="V469" s="4" t="n"/>
     </row>
     <row r="470">
       <c r="A470" s="4" t="n"/>
@@ -7785,6 +8422,7 @@
       <c r="S470" s="4" t="n"/>
       <c r="T470" s="4" t="n"/>
       <c r="U470" s="4" t="n"/>
+      <c r="V470" s="4" t="n"/>
     </row>
     <row r="471">
       <c r="A471" s="4" t="n"/>
@@ -7799,6 +8437,7 @@
       <c r="S471" s="4" t="n"/>
       <c r="T471" s="4" t="n"/>
       <c r="U471" s="4" t="n"/>
+      <c r="V471" s="4" t="n"/>
     </row>
     <row r="472">
       <c r="A472" s="4" t="n"/>
@@ -7813,6 +8452,7 @@
       <c r="S472" s="4" t="n"/>
       <c r="T472" s="4" t="n"/>
       <c r="U472" s="4" t="n"/>
+      <c r="V472" s="4" t="n"/>
     </row>
     <row r="473">
       <c r="A473" s="4" t="n"/>
@@ -7827,6 +8467,7 @@
       <c r="S473" s="4" t="n"/>
       <c r="T473" s="4" t="n"/>
       <c r="U473" s="4" t="n"/>
+      <c r="V473" s="4" t="n"/>
     </row>
     <row r="474">
       <c r="A474" s="4" t="n"/>
@@ -7841,6 +8482,7 @@
       <c r="S474" s="4" t="n"/>
       <c r="T474" s="4" t="n"/>
       <c r="U474" s="4" t="n"/>
+      <c r="V474" s="4" t="n"/>
     </row>
     <row r="475">
       <c r="A475" s="4" t="n"/>
@@ -7855,6 +8497,7 @@
       <c r="S475" s="4" t="n"/>
       <c r="T475" s="4" t="n"/>
       <c r="U475" s="4" t="n"/>
+      <c r="V475" s="4" t="n"/>
     </row>
     <row r="476">
       <c r="A476" s="4" t="n"/>
@@ -7869,6 +8512,7 @@
       <c r="S476" s="4" t="n"/>
       <c r="T476" s="4" t="n"/>
       <c r="U476" s="4" t="n"/>
+      <c r="V476" s="4" t="n"/>
     </row>
     <row r="477">
       <c r="A477" s="4" t="n"/>
@@ -7883,6 +8527,7 @@
       <c r="S477" s="4" t="n"/>
       <c r="T477" s="4" t="n"/>
       <c r="U477" s="4" t="n"/>
+      <c r="V477" s="4" t="n"/>
     </row>
     <row r="478">
       <c r="A478" s="4" t="n"/>
@@ -7897,6 +8542,7 @@
       <c r="S478" s="4" t="n"/>
       <c r="T478" s="4" t="n"/>
       <c r="U478" s="4" t="n"/>
+      <c r="V478" s="4" t="n"/>
     </row>
     <row r="479">
       <c r="A479" s="4" t="n"/>
@@ -7911,6 +8557,7 @@
       <c r="S479" s="4" t="n"/>
       <c r="T479" s="4" t="n"/>
       <c r="U479" s="4" t="n"/>
+      <c r="V479" s="4" t="n"/>
     </row>
     <row r="480">
       <c r="A480" s="4" t="n"/>
@@ -7925,6 +8572,7 @@
       <c r="S480" s="4" t="n"/>
       <c r="T480" s="4" t="n"/>
       <c r="U480" s="4" t="n"/>
+      <c r="V480" s="4" t="n"/>
     </row>
     <row r="481">
       <c r="A481" s="4" t="n"/>
@@ -7939,6 +8587,7 @@
       <c r="S481" s="4" t="n"/>
       <c r="T481" s="4" t="n"/>
       <c r="U481" s="4" t="n"/>
+      <c r="V481" s="4" t="n"/>
     </row>
     <row r="482">
       <c r="A482" s="4" t="n"/>
@@ -7953,6 +8602,7 @@
       <c r="S482" s="4" t="n"/>
       <c r="T482" s="4" t="n"/>
       <c r="U482" s="4" t="n"/>
+      <c r="V482" s="4" t="n"/>
     </row>
     <row r="483">
       <c r="A483" s="4" t="n"/>
@@ -7967,6 +8617,7 @@
       <c r="S483" s="4" t="n"/>
       <c r="T483" s="4" t="n"/>
       <c r="U483" s="4" t="n"/>
+      <c r="V483" s="4" t="n"/>
     </row>
     <row r="484">
       <c r="A484" s="4" t="n"/>
@@ -7981,6 +8632,7 @@
       <c r="S484" s="4" t="n"/>
       <c r="T484" s="4" t="n"/>
       <c r="U484" s="4" t="n"/>
+      <c r="V484" s="4" t="n"/>
     </row>
     <row r="485">
       <c r="A485" s="4" t="n"/>
@@ -7995,6 +8647,7 @@
       <c r="S485" s="4" t="n"/>
       <c r="T485" s="4" t="n"/>
       <c r="U485" s="4" t="n"/>
+      <c r="V485" s="4" t="n"/>
     </row>
     <row r="486">
       <c r="A486" s="4" t="n"/>
@@ -8009,6 +8662,7 @@
       <c r="S486" s="4" t="n"/>
       <c r="T486" s="4" t="n"/>
       <c r="U486" s="4" t="n"/>
+      <c r="V486" s="4" t="n"/>
     </row>
     <row r="487">
       <c r="A487" s="4" t="n"/>
@@ -8023,6 +8677,7 @@
       <c r="S487" s="4" t="n"/>
       <c r="T487" s="4" t="n"/>
       <c r="U487" s="4" t="n"/>
+      <c r="V487" s="4" t="n"/>
     </row>
     <row r="488">
       <c r="A488" s="4" t="n"/>
@@ -8037,6 +8692,7 @@
       <c r="S488" s="4" t="n"/>
       <c r="T488" s="4" t="n"/>
       <c r="U488" s="4" t="n"/>
+      <c r="V488" s="4" t="n"/>
     </row>
     <row r="489">
       <c r="A489" s="4" t="n"/>
@@ -8051,6 +8707,7 @@
       <c r="S489" s="4" t="n"/>
       <c r="T489" s="4" t="n"/>
       <c r="U489" s="4" t="n"/>
+      <c r="V489" s="4" t="n"/>
     </row>
     <row r="490">
       <c r="A490" s="4" t="n"/>
@@ -8065,6 +8722,7 @@
       <c r="S490" s="4" t="n"/>
       <c r="T490" s="4" t="n"/>
       <c r="U490" s="4" t="n"/>
+      <c r="V490" s="4" t="n"/>
     </row>
     <row r="491">
       <c r="A491" s="4" t="n"/>
@@ -8079,6 +8737,7 @@
       <c r="S491" s="4" t="n"/>
       <c r="T491" s="4" t="n"/>
       <c r="U491" s="4" t="n"/>
+      <c r="V491" s="4" t="n"/>
     </row>
     <row r="492">
       <c r="A492" s="4" t="n"/>
@@ -8093,6 +8752,7 @@
       <c r="S492" s="4" t="n"/>
       <c r="T492" s="4" t="n"/>
       <c r="U492" s="4" t="n"/>
+      <c r="V492" s="4" t="n"/>
     </row>
     <row r="493">
       <c r="A493" s="4" t="n"/>
@@ -8107,6 +8767,7 @@
       <c r="S493" s="4" t="n"/>
       <c r="T493" s="4" t="n"/>
       <c r="U493" s="4" t="n"/>
+      <c r="V493" s="4" t="n"/>
     </row>
     <row r="494">
       <c r="A494" s="4" t="n"/>
@@ -8121,6 +8782,7 @@
       <c r="S494" s="4" t="n"/>
       <c r="T494" s="4" t="n"/>
       <c r="U494" s="4" t="n"/>
+      <c r="V494" s="4" t="n"/>
     </row>
     <row r="495">
       <c r="A495" s="4" t="n"/>
@@ -8135,6 +8797,7 @@
       <c r="S495" s="4" t="n"/>
       <c r="T495" s="4" t="n"/>
       <c r="U495" s="4" t="n"/>
+      <c r="V495" s="4" t="n"/>
     </row>
     <row r="496">
       <c r="A496" s="4" t="n"/>
@@ -8149,6 +8812,7 @@
       <c r="S496" s="4" t="n"/>
       <c r="T496" s="4" t="n"/>
       <c r="U496" s="4" t="n"/>
+      <c r="V496" s="4" t="n"/>
     </row>
     <row r="497">
       <c r="A497" s="4" t="n"/>
@@ -8163,6 +8827,7 @@
       <c r="S497" s="4" t="n"/>
       <c r="T497" s="4" t="n"/>
       <c r="U497" s="4" t="n"/>
+      <c r="V497" s="4" t="n"/>
     </row>
     <row r="498">
       <c r="A498" s="4" t="n"/>
@@ -8177,6 +8842,7 @@
       <c r="S498" s="4" t="n"/>
       <c r="T498" s="4" t="n"/>
       <c r="U498" s="4" t="n"/>
+      <c r="V498" s="4" t="n"/>
     </row>
     <row r="499">
       <c r="A499" s="4" t="n"/>
@@ -8191,6 +8857,7 @@
       <c r="S499" s="4" t="n"/>
       <c r="T499" s="4" t="n"/>
       <c r="U499" s="4" t="n"/>
+      <c r="V499" s="4" t="n"/>
     </row>
     <row r="500">
       <c r="A500" s="4" t="n"/>
@@ -8205,14 +8872,18 @@
       <c r="S500" s="4" t="n"/>
       <c r="T500" s="4" t="n"/>
       <c r="U500" s="4" t="n"/>
+      <c r="V500" s="4" t="n"/>
     </row>
   </sheetData>
-  <dataValidations count="2">
+  <dataValidations count="3">
     <dataValidation sqref="F2:F500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Use um destes valores: estavel, transitorio, partida, parada" type="list">
       <formula1>"estavel,transitorio,partida,parada"</formula1>
     </dataValidation>
     <dataValidation sqref="U2:U500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Use um destes valores: sintetico, publico, real" type="list">
       <formula1>"sintetico,publico,real"</formula1>
+    </dataValidation>
+    <dataValidation sqref="V2:V500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Use um destes valores: saturado_seco, umido, superaquecido" type="list">
+      <formula1>"saturado_seco,umido,superaquecido"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
fix: audita rotas adaptativas e preserva fronteiras fisicas
</commit_message>
<xml_diff>
--- a/templates/planilha_modelo_euler.xlsx
+++ b/templates/planilha_modelo_euler.xlsx
@@ -393,8 +393,36 @@
     </comment>
     <comment ref="AI1" authorId="0" shapeId="0">
       <text>
-        <t>Pressão da água no mesmo ponto da temperatura t_agua_alim_c, usada como referência na energia da purga.
+        <t>Pressão da água no mesmo ponto da temperatura t_agua_alim_c, usada na purga e no balanço por vazões do historiador.
 Unidade: bar manométrico
+Opcional</t>
+      </text>
+    </comment>
+    <comment ref="AJ1" authorId="0" shapeId="0">
+      <text>
+        <t>Vazão instantânea de vapor. Permite rota por historiador sem depender do totalizador.
+Unidade: t/h
+Opcional</t>
+      </text>
+    </comment>
+    <comment ref="AK1" authorId="0" shapeId="0">
+      <text>
+        <t>Vazão mássica instantânea de combustível na mesma base do PCI informado.
+Unidade: kg/h
+Opcional</t>
+      </text>
+    </comment>
+    <comment ref="AL1" authorId="0" shapeId="0">
+      <text>
+        <t>PCI correspondente ao combustível na condição/base em que a vazão mássica é medida.
+Unidade: MJ/kg como recebido
+Opcional</t>
+      </text>
+    </comment>
+    <comment ref="AM1" authorId="0" shapeId="0">
+      <text>
+        <t>Potência térmica de entrada do combustível já fornecida pelo sistema da planta.
+Unidade: MW térmico
 Opcional</t>
       </text>
     </comment>
@@ -1121,7 +1149,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AI500"/>
+  <dimension ref="A1:AM500"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -1159,6 +1187,10 @@
     <col width="17" customWidth="1" min="33" max="33"/>
     <col width="16" customWidth="1" min="34" max="34"/>
     <col width="29" customWidth="1" min="35" max="35"/>
+    <col width="19" customWidth="1" min="36" max="36"/>
+    <col width="26" customWidth="1" min="37" max="37"/>
+    <col width="25" customWidth="1" min="38" max="38"/>
+    <col width="27" customWidth="1" min="39" max="39"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1337,6 +1369,26 @@
           <t>p_agua_referencia_bar_man</t>
         </is>
       </c>
+      <c r="AJ1" s="3" t="inlineStr">
+        <is>
+          <t>vazao_vapor_t_h</t>
+        </is>
+      </c>
+      <c r="AK1" s="3" t="inlineStr">
+        <is>
+          <t>vazao_combustivel_kg_h</t>
+        </is>
+      </c>
+      <c r="AL1" s="3" t="inlineStr">
+        <is>
+          <t>pci_combustivel_mj_kg</t>
+        </is>
+      </c>
+      <c r="AM1" s="3" t="inlineStr">
+        <is>
+          <t>potencia_combustivel_mw</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="4" t="inlineStr">

</xml_diff>